<commit_message>
feat: add free sources and direct evidence links
</commit_message>
<xml_diff>
--- a/output/precedent_transactions.xlsx
+++ b/output/precedent_transactions.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal Dashboard" sheetId="1" r:id="Rdd12d12ff2da4122"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="2" r:id="R328d3bbdd89c4d60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal Card" sheetId="3" r:id="R62e5697d724f4edb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; QA" sheetId="4" r:id="Rcd48572823e84eb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal Dashboard" sheetId="1" r:id="R209f00ac58ba4bfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="2" r:id="Rf51a889b1a7f4027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal Card" sheetId="3" r:id="R6b6d26b547cf48c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; QA" sheetId="4" r:id="R9e0c98700761402c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -318,7 +318,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PrecedentTransactionsTable" displayName="PrecedentTransactionsTable" ref="A6:AC43" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PrecedentTransactionsTable" displayName="PrecedentTransactionsTable" ref="A6:AC56" headerRowCount="1">
   <x:tableColumns count="29">
     <x:tableColumn id="1" name="Deal ID"/>
     <x:tableColumn id="2" name="Announced Date"/>
@@ -624,31 +624,31 @@
     <x:row r="7" ht="32" customHeight="1">
       <x:c r="A7" s="28" t="n">
         <x:f>COUNTA('Precedent Transactions'!$A$7:$A$506)</x:f>
-        <x:v>37</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B7" s="29" t="n">
         <x:f>COUNTIF('Precedent Transactions'!$C$7:$C$506,"M&amp;A")</x:f>
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C7" s="29" t="n">
         <x:f>COUNTIF('Precedent Transactions'!$C$7:$C$506,"ECM")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D7" s="29" t="n">
         <x:f>COUNTIF('Precedent Transactions'!$C$7:$C$506,"DCM")</x:f>
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E7" s="31" t="n">
         <x:f>SUM('Precedent Transactions'!$I$7:$I$506)</x:f>
-        <x:v>252300000000</x:v>
+        <x:v>589300000000</x:v>
       </x:c>
       <x:c r="F7" s="29" t="n">
         <x:f>COUNTIF('Precedent Transactions'!$W$7:$W$506,"&gt;=7")</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G7" s="29" t="n">
         <x:f>COUNTBLANK('Precedent Transactions'!$I$7:$I$506)-COUNTBLANK('Precedent Transactions'!$A$7:$A$506)</x:f>
-        <x:v>26</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="H7" s="30" t="str">
         <x:f>'Sources &amp; QA'!$F$31</x:f>
@@ -739,26 +739,28 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="36" t="n">
-        <x:v>46199</x:v>
+        <x:v>46201</x:v>
       </x:c>
       <x:c r="B19" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>MTSS</x:v>
       </x:c>
       <x:c r="E19" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
-      <x:c r="F19" s="37"/>
+      <x:c r="F19" s="37" t="n">
+        <x:v>20000000000</x:v>
+      </x:c>
       <x:c r="G19" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="H19" t="str">
-        <x:v>MOEX disclosure</x:v>
+        <x:v>MTS Investor Relations</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -772,7 +774,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="D20" t="str">
-        <x:v>О регистрации проспекта биржевых облигаций</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="E20" t="str">
         <x:v>Not applicable</x:v>
@@ -796,7 +798,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="D21" t="str">
-        <x:v>О регистрации изменений в эмиссионные документы</x:v>
+        <x:v>О регистрации проспекта биржевых облигаций</x:v>
       </x:c>
       <x:c r="E21" t="str">
         <x:v>Not applicable</x:v>
@@ -820,7 +822,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="D22" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>О регистрации изменений в эмиссионные документы</x:v>
       </x:c>
       <x:c r="E22" t="str">
         <x:v>Not applicable</x:v>
@@ -868,7 +870,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="D24" t="str">
-        <x:v>О проведении выкупа облигаций с 29 июня по 03 июля 2026 года</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="E24" t="str">
         <x:v>Not applicable</x:v>
@@ -892,7 +894,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="D25" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>О проведении выкупа облигаций с 29 июня по 03 июля 2026 года</x:v>
       </x:c>
       <x:c r="E25" t="str">
         <x:v>Not applicable</x:v>
@@ -907,80 +909,78 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="36" t="n">
-        <x:v>46197</x:v>
+        <x:v>46199</x:v>
       </x:c>
       <x:c r="B26" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>Announced</x:v>
+        <x:v>Reported</x:v>
       </x:c>
       <x:c r="D26" t="str">
-        <x:v>Selectel</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="E26" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
-      <x:c r="F26" s="37" t="n">
-        <x:v>5000000000</x:v>
-      </x:c>
+      <x:c r="F26" s="37"/>
       <x:c r="G26" t="str">
-        <x:v>RUB</x:v>
+        <x:v>NOT DISCLOSED</x:v>
       </x:c>
       <x:c r="H26" t="str">
-        <x:v>ComNews.ru</x:v>
+        <x:v>MOEX disclosure</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="36" t="n">
-        <x:v>46192</x:v>
+        <x:v>46197</x:v>
       </x:c>
       <x:c r="B27" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>Issued</x:v>
+        <x:v>Announced</x:v>
       </x:c>
       <x:c r="D27" t="str">
-        <x:v>Yandex</x:v>
+        <x:v>Selectel</x:v>
       </x:c>
       <x:c r="E27" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="F27" s="37" t="n">
-        <x:v>60000000000</x:v>
+        <x:v>5000000000</x:v>
       </x:c>
       <x:c r="G27" t="str">
         <x:v>RUB</x:v>
       </x:c>
       <x:c r="H27" t="str">
-        <x:v>Yandex Investor Relations</x:v>
+        <x:v>ComNews.ru</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="36" t="n">
-        <x:v>46183</x:v>
+        <x:v>46192</x:v>
       </x:c>
       <x:c r="B28" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Issued</x:v>
       </x:c>
       <x:c r="D28" t="str">
-        <x:v>Норникель</x:v>
+        <x:v>Yandex</x:v>
       </x:c>
       <x:c r="E28" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="F28" s="37" t="n">
-        <x:v>3000000000</x:v>
+        <x:v>60000000000</x:v>
       </x:c>
       <x:c r="G28" t="str">
         <x:v>RUB</x:v>
       </x:c>
       <x:c r="H28" t="str">
-        <x:v>Интерфакс</x:v>
+        <x:v>Yandex Investor Relations</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1220,19 +1220,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="41" t="str">
-        <x:v>DL-moex-101492</x:v>
+        <x:v>DL-4d8f7bcb385b1c88</x:v>
       </x:c>
       <x:c r="B7" s="43" t="n">
-        <x:v>46199</x:v>
+        <x:v>46201</x:v>
       </x:c>
       <x:c r="C7" s="41" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="D7" s="41" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E7" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>MTSS</x:v>
       </x:c>
       <x:c r="F7" s="41" t="str">
         <x:v>Not applicable</x:v>
@@ -1243,10 +1243,12 @@
       <x:c r="H7" s="41" t="str">
         <x:v>Russia</x:v>
       </x:c>
-      <x:c r="I7" s="44"/>
+      <x:c r="I7" s="44" t="n">
+        <x:v>20000000000</x:v>
+      </x:c>
       <x:c r="J7" s="44"/>
       <x:c r="K7" s="41" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="L7" s="45"/>
       <x:c r="M7" s="41" t="str">
@@ -1276,20 +1278,20 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W7" s="41" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="X7" s="41" t="str">
         <x:v>confirmed</x:v>
       </x:c>
       <x:c r="Y7" s="41" t="str"/>
       <x:c r="Z7" s="41" t="str">
-        <x:v>MOEX disclosure</x:v>
+        <x:v>MTS Investor Relations</x:v>
       </x:c>
       <x:c r="AA7" s="41" t="str">
-        <x:v>https://www.moex.com/n101492</x:v>
+        <x:v>https://ir.mts.ru/news_and_events/corporate_releases/details/742414</x:v>
       </x:c>
       <x:c r="AB7" s="41" t="str">
-        <x:v>О регистрации выпуска биржевых облигаций, о включении его в Список ценных бумаг, допущенных к торгам, и о присвоении указанным биржевым облигациям регистрационного номера</x:v>
+        <x:v>МТС успешно закрыла книгу биржевых облигаций 003Р-03 на 20 млрд руб.</x:v>
       </x:c>
       <x:c r="AC7" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1297,7 +1299,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="41" t="str">
-        <x:v>DL-moex-101473</x:v>
+        <x:v>DL-moex-101492</x:v>
       </x:c>
       <x:c r="B8" s="43" t="n">
         <x:v>46199</x:v>
@@ -1309,7 +1311,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E8" s="41" t="str">
-        <x:v>О регистрации проспекта биржевых облигаций</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F8" s="41" t="str">
         <x:v>Not applicable</x:v>
@@ -1363,10 +1365,10 @@
         <x:v>MOEX disclosure</x:v>
       </x:c>
       <x:c r="AA8" s="41" t="str">
-        <x:v>https://www.moex.com/n101473</x:v>
+        <x:v>https://www.moex.com/n101492</x:v>
       </x:c>
       <x:c r="AB8" s="41" t="str">
-        <x:v>О регистрации проспекта биржевых облигаций</x:v>
+        <x:v>О регистрации выпуска биржевых облигаций, о включении его в Список ценных бумаг, допущенных к торгам, и о присвоении указанным биржевым облигациям регистрационного номера</x:v>
       </x:c>
       <x:c r="AC8" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1374,7 +1376,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="41" t="str">
-        <x:v>DL-moex-101468</x:v>
+        <x:v>DL-moex-101473</x:v>
       </x:c>
       <x:c r="B9" s="43" t="n">
         <x:v>46199</x:v>
@@ -1386,7 +1388,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E9" s="41" t="str">
-        <x:v>О регистрации изменений в эмиссионные документы</x:v>
+        <x:v>О регистрации проспекта биржевых облигаций</x:v>
       </x:c>
       <x:c r="F9" s="41" t="str">
         <x:v>Not applicable</x:v>
@@ -1440,10 +1442,10 @@
         <x:v>MOEX disclosure</x:v>
       </x:c>
       <x:c r="AA9" s="41" t="str">
-        <x:v>https://www.moex.com/n101468</x:v>
+        <x:v>https://www.moex.com/n101473</x:v>
       </x:c>
       <x:c r="AB9" s="41" t="str">
-        <x:v>О регистрации изменений в эмиссионные документы</x:v>
+        <x:v>О регистрации проспекта биржевых облигаций</x:v>
       </x:c>
       <x:c r="AC9" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1451,7 +1453,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="41" t="str">
-        <x:v>DL-moex-101457</x:v>
+        <x:v>DL-moex-101468</x:v>
       </x:c>
       <x:c r="B10" s="43" t="n">
         <x:v>46199</x:v>
@@ -1463,16 +1465,16 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E10" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>О регистрации изменений в эмиссионные документы</x:v>
       </x:c>
       <x:c r="F10" s="41" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G10" s="41" t="str">
-        <x:v>Financials</x:v>
+        <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H10" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Russia</x:v>
       </x:c>
       <x:c r="I10" s="44"/>
       <x:c r="J10" s="44"/>
@@ -1517,10 +1519,10 @@
         <x:v>MOEX disclosure</x:v>
       </x:c>
       <x:c r="AA10" s="41" t="str">
-        <x:v>https://www.moex.com/n101457</x:v>
+        <x:v>https://www.moex.com/n101468</x:v>
       </x:c>
       <x:c r="AB10" s="41" t="str">
-        <x:v>О порядке сбора заявок и заключения сделок при размещении облигаций серии Б-1-403 Банк ВТБ (публичное акционерное общество) с 29 июня 2026 года</x:v>
+        <x:v>О регистрации изменений в эмиссионные документы</x:v>
       </x:c>
       <x:c r="AC10" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1528,7 +1530,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="41" t="str">
-        <x:v>DL-moex-101454</x:v>
+        <x:v>DL-moex-101457</x:v>
       </x:c>
       <x:c r="B11" s="43" t="n">
         <x:v>46199</x:v>
@@ -1549,16 +1551,14 @@
         <x:v>Financials</x:v>
       </x:c>
       <x:c r="H11" s="41" t="str">
-        <x:v>Russia</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="I11" s="44"/>
       <x:c r="J11" s="44"/>
       <x:c r="K11" s="41" t="str">
         <x:v>NOT DISCLOSED</x:v>
       </x:c>
-      <x:c r="L11" s="45" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="L11" s="45"/>
       <x:c r="M11" s="41" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
@@ -1596,10 +1596,10 @@
         <x:v>MOEX disclosure</x:v>
       </x:c>
       <x:c r="AA11" s="41" t="str">
-        <x:v>https://www.moex.com/n101454</x:v>
+        <x:v>https://www.moex.com/n101457</x:v>
       </x:c>
       <x:c r="AB11" s="41" t="str">
-        <x:v>О порядке приобретения облигаций серии 001P-04 ООО "АРЕНЗА-ПРО" с 29 июня 2026 год</x:v>
+        <x:v>О порядке сбора заявок и заключения сделок при размещении облигаций серии Б-1-403 Банк ВТБ (публичное акционерное общество) с 29 июня 2026 года</x:v>
       </x:c>
       <x:c r="AC11" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1607,7 +1607,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="41" t="str">
-        <x:v>DL-moex-101451</x:v>
+        <x:v>DL-moex-101454</x:v>
       </x:c>
       <x:c r="B12" s="43" t="n">
         <x:v>46199</x:v>
@@ -1619,23 +1619,25 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E12" s="41" t="str">
-        <x:v>О проведении выкупа облигаций с 29 июня по 03 июля 2026 года</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F12" s="41" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G12" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Financials</x:v>
       </x:c>
       <x:c r="H12" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Russia</x:v>
       </x:c>
       <x:c r="I12" s="44"/>
       <x:c r="J12" s="44"/>
       <x:c r="K12" s="41" t="str">
         <x:v>NOT DISCLOSED</x:v>
       </x:c>
-      <x:c r="L12" s="45"/>
+      <x:c r="L12" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="M12" s="41" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
@@ -1673,10 +1675,10 @@
         <x:v>MOEX disclosure</x:v>
       </x:c>
       <x:c r="AA12" s="41" t="str">
-        <x:v>https://www.moex.com/n101451</x:v>
+        <x:v>https://www.moex.com/n101454</x:v>
       </x:c>
       <x:c r="AB12" s="41" t="str">
-        <x:v>О проведении выкупа облигаций с 29 июня по 03 июля 2026 года</x:v>
+        <x:v>О порядке приобретения облигаций серии 001P-04 ООО "АРЕНЗА-ПРО" с 29 июня 2026 год</x:v>
       </x:c>
       <x:c r="AC12" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1684,7 +1686,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="41" t="str">
-        <x:v>DL-moex-101450</x:v>
+        <x:v>DL-moex-101451</x:v>
       </x:c>
       <x:c r="B13" s="43" t="n">
         <x:v>46199</x:v>
@@ -1696,7 +1698,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E13" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>О проведении выкупа облигаций с 29 июня по 03 июля 2026 года</x:v>
       </x:c>
       <x:c r="F13" s="41" t="str">
         <x:v>Not applicable</x:v>
@@ -1705,7 +1707,7 @@
         <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H13" s="41" t="str">
-        <x:v>Russia</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="I13" s="44"/>
       <x:c r="J13" s="44"/>
@@ -1750,10 +1752,10 @@
         <x:v>MOEX disclosure</x:v>
       </x:c>
       <x:c r="AA13" s="41" t="str">
-        <x:v>https://www.moex.com/n101450</x:v>
+        <x:v>https://www.moex.com/n101451</x:v>
       </x:c>
       <x:c r="AB13" s="41" t="str">
-        <x:v>Дополнительные условия проведения торгов по выкупу облигаций серии 003Р-02 ООО "Концерн "РОССИУМ" 26 июня 2026 года</x:v>
+        <x:v>О проведении выкупа облигаций с 29 июня по 03 июля 2026 года</x:v>
       </x:c>
       <x:c r="AC13" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1761,19 +1763,19 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="41" t="str">
-        <x:v>DL-bec65812ff9fcfae</x:v>
+        <x:v>DL-moex-101450</x:v>
       </x:c>
       <x:c r="B14" s="43" t="n">
-        <x:v>46197</x:v>
+        <x:v>46199</x:v>
       </x:c>
       <x:c r="C14" s="41" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="D14" s="41" t="str">
-        <x:v>Announced</x:v>
+        <x:v>Reported</x:v>
       </x:c>
       <x:c r="E14" s="41" t="str">
-        <x:v>Selectel</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F14" s="41" t="str">
         <x:v>Not applicable</x:v>
@@ -1784,20 +1786,26 @@
       <x:c r="H14" s="41" t="str">
         <x:v>Russia</x:v>
       </x:c>
-      <x:c r="I14" s="44" t="n">
-        <x:v>5000000000</x:v>
-      </x:c>
+      <x:c r="I14" s="44"/>
       <x:c r="J14" s="44"/>
       <x:c r="K14" s="41" t="str">
-        <x:v>RUB</x:v>
+        <x:v>NOT DISCLOSED</x:v>
       </x:c>
       <x:c r="L14" s="45"/>
-      <x:c r="M14" s="41"/>
-      <x:c r="N14" s="41"/>
+      <x:c r="M14" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N14" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
       <x:c r="O14" s="44"/>
       <x:c r="P14" s="44"/>
-      <x:c r="Q14" s="41"/>
-      <x:c r="R14" s="41"/>
+      <x:c r="Q14" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R14" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
       <x:c r="S14" s="46" t="str">
         <x:f>IFERROR(IF(AND($J14&gt;0,$O14&gt;0,$K14=$R14),$J14/$O14,""),"")</x:f>
       </x:c>
@@ -1808,23 +1816,23 @@
         <x:v>Bonds</x:v>
       </x:c>
       <x:c r="V14" s="41" t="str">
-        <x:v>рефинансирования и инвестиций</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W14" s="41" t="n">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="X14" s="41" t="str">
-        <x:v>unverified</x:v>
+        <x:v>confirmed</x:v>
       </x:c>
       <x:c r="Y14" s="41" t="str"/>
       <x:c r="Z14" s="41" t="str">
-        <x:v>ComNews.ru</x:v>
+        <x:v>MOEX disclosure</x:v>
       </x:c>
       <x:c r="AA14" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMi1AFBVV95cUxOZ0FzQTE1TUJkMGFCVjZuNTBGY0JwNTZBaS16Wnl0NW9XSXBmNFlTRUJacXFlV0tYdUxpUTZTWVhNWk4wYll4a3dZZEU2ZFYzZ2d6T2YwUl85bGlXZGRpN3NiTXJwcnExdzBVVkx6YWV1eExnOFJlcmlDb21UTG5KQWozVTNhX0VwNDVmdnFYTEQwcFpENjdHMjhEX01fTERSUHpsNkE2a3FESkdwbzEzbGRsXzB6MWFlVW80Ri1fa0JYdDVKNEhMZml2WmtiSWYyV2tuZA?oc=5</x:v>
+        <x:v>https://www.moex.com/n101450</x:v>
       </x:c>
       <x:c r="AB14" s="41" t="str">
-        <x:v>Selectel разместит облигации на 5 млрд руб. для рефинансирования и инвестиций - ComNews.ru</x:v>
+        <x:v>Дополнительные условия проведения торгов по выкупу облигаций серии 003Р-02 ООО "Концерн "РОССИУМ" 26 июня 2026 года</x:v>
       </x:c>
       <x:c r="AC14" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1832,51 +1840,43 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="41" t="str">
-        <x:v>DL-48bd4fc3fa031e6c</x:v>
+        <x:v>DL-bec65812ff9fcfae</x:v>
       </x:c>
       <x:c r="B15" s="43" t="n">
-        <x:v>46192</x:v>
+        <x:v>46197</x:v>
       </x:c>
       <x:c r="C15" s="41" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="D15" s="41" t="str">
-        <x:v>Issued</x:v>
+        <x:v>Announced</x:v>
       </x:c>
       <x:c r="E15" s="41" t="str">
-        <x:v>Yandex</x:v>
+        <x:v>Selectel</x:v>
       </x:c>
       <x:c r="F15" s="41" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G15" s="41" t="str">
-        <x:v>Technology</x:v>
+        <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H15" s="41" t="str">
         <x:v>Russia</x:v>
       </x:c>
       <x:c r="I15" s="44" t="n">
-        <x:v>60000000000</x:v>
+        <x:v>5000000000</x:v>
       </x:c>
       <x:c r="J15" s="44"/>
       <x:c r="K15" s="41" t="str">
         <x:v>RUB</x:v>
       </x:c>
       <x:c r="L15" s="45"/>
-      <x:c r="M15" s="41" t="str">
-        <x:v>Not applicable</x:v>
-      </x:c>
-      <x:c r="N15" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
+      <x:c r="M15" s="41"/>
+      <x:c r="N15" s="41"/>
       <x:c r="O15" s="44"/>
       <x:c r="P15" s="44"/>
-      <x:c r="Q15" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
-      <x:c r="R15" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
+      <x:c r="Q15" s="41"/>
+      <x:c r="R15" s="41"/>
       <x:c r="S15" s="46" t="str">
         <x:f>IFERROR(IF(AND($J15&gt;0,$O15&gt;0,$K15=$R15),$J15/$O15,""),"")</x:f>
       </x:c>
@@ -1887,25 +1887,23 @@
         <x:v>Bonds</x:v>
       </x:c>
       <x:c r="V15" s="41" t="str">
-        <x:v>частных инвесторов Яндекса содержит информацию про бизнесы и технологии компании, а также географию присутствия, финансовые результаты, важные новости и многое другое о компании и её рынках</x:v>
+        <x:v>рефинансирования и инвестиций</x:v>
       </x:c>
       <x:c r="W15" s="41" t="n">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X15" s="41" t="str">
-        <x:v>confirmed</x:v>
-      </x:c>
-      <x:c r="Y15" s="41" t="str">
-        <x:v>YDEX</x:v>
-      </x:c>
+        <x:v>unverified</x:v>
+      </x:c>
+      <x:c r="Y15" s="41" t="str"/>
       <x:c r="Z15" s="41" t="str">
-        <x:v>Yandex Investor Relations</x:v>
+        <x:v>ComNews.ru</x:v>
       </x:c>
       <x:c r="AA15" s="41" t="str">
-        <x:v>https://ir.yandex.ru/press-releases?year=2026&amp;id=19-06-2026-03</x:v>
+        <x:v>https://www.comnews.ru/content/246003/2026-06-25/2026-w26/1008/selectel-razmestit-obligacii-5-mlrd-rub-dlya-refinansirovaniya-i-investiciy</x:v>
       </x:c>
       <x:c r="AB15" s="41" t="str">
-        <x:v>Яндекс разместил два выпуска биржевых облигаций на общую сумму 60 млрд рублей</x:v>
+        <x:v>Selectel разместит облигации на 5 млрд руб. для рефинансирования и инвестиций - ComNews.ru</x:v>
       </x:c>
       <x:c r="AC15" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1913,31 +1911,31 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="41" t="str">
-        <x:v>DL-9092ffd6a36a0a81</x:v>
+        <x:v>DL-7a721642a53e0f1d</x:v>
       </x:c>
       <x:c r="B16" s="43" t="n">
-        <x:v>46183</x:v>
+        <x:v>46192</x:v>
       </x:c>
       <x:c r="C16" s="41" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="D16" s="41" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Issued</x:v>
       </x:c>
       <x:c r="E16" s="41" t="str">
-        <x:v>Норникель</x:v>
+        <x:v>Yandex</x:v>
       </x:c>
       <x:c r="F16" s="41" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G16" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Technology</x:v>
       </x:c>
       <x:c r="H16" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Russia</x:v>
       </x:c>
       <x:c r="I16" s="44" t="n">
-        <x:v>3000000000</x:v>
+        <x:v>60000000000</x:v>
       </x:c>
       <x:c r="J16" s="44"/>
       <x:c r="K16" s="41" t="str">
@@ -1968,23 +1966,25 @@
         <x:v>Bonds</x:v>
       </x:c>
       <x:c r="V16" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>частных инвесторов Яндекса содержит информацию про бизнесы и технологии компании, а также географию присутствия, финансовые результаты, важные новости и многое другое о компании и её рынках</x:v>
       </x:c>
       <x:c r="W16" s="41" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="X16" s="41" t="str">
-        <x:v>unverified</x:v>
-      </x:c>
-      <x:c r="Y16" s="41" t="str"/>
+        <x:v>confirmed</x:v>
+      </x:c>
+      <x:c r="Y16" s="41" t="str">
+        <x:v>YDEX</x:v>
+      </x:c>
       <x:c r="Z16" s="41" t="str">
-        <x:v>Интерфакс</x:v>
+        <x:v>Yandex Investor Relations</x:v>
       </x:c>
       <x:c r="AA16" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE1YcWRJT1pJS3JQYUlDcVBxQmRrd2JFXzdidEJQMkRoTFVIRlBDUnQ5ZjNSMFZGamhRQ1hoTXFwaUVQMW1PZldFWWhvSzdOdmtSQnfSAUtBVV95cUxQWkQ5UHd5NFJieHBKUTVCZURpX1dEWmM4a2FnOXJ3aUREYi04ZGFUclFMNUxBdU1EMFVYWUU4MlhCaXJfTy1NZlVNXzg?oc=5</x:v>
+        <x:v>https://ir.yandex.ru/press-releases?year=2026&amp;id=19-06-2026-03</x:v>
       </x:c>
       <x:c r="AB16" s="41" t="str">
-        <x:v>"Норникель" зафиксировал объем размещения облигаций на уровне 3 млрд юаней - Интерфакс</x:v>
+        <x:v>Яндекс разместил два выпуска биржевых облигаций на общую сумму 60 млрд рублей</x:v>
       </x:c>
       <x:c r="AC16" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -1992,10 +1992,10 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="41" t="str">
-        <x:v>DL-f71ff729dc9f5af4</x:v>
+        <x:v>DL-9092ffd6a36a0a81</x:v>
       </x:c>
       <x:c r="B17" s="43" t="n">
-        <x:v>46181</x:v>
+        <x:v>46183</x:v>
       </x:c>
       <x:c r="C17" s="41" t="str">
         <x:v>DCM</x:v>
@@ -2004,7 +2004,7 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E17" s="41" t="str">
-        <x:v>Yandex</x:v>
+        <x:v>Норникель</x:v>
       </x:c>
       <x:c r="F17" s="41" t="str">
         <x:v>Not applicable</x:v>
@@ -2015,10 +2015,12 @@
       <x:c r="H17" s="41" t="str">
         <x:v>Not disclosed</x:v>
       </x:c>
-      <x:c r="I17" s="44"/>
+      <x:c r="I17" s="44" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
       <x:c r="J17" s="44"/>
       <x:c r="K17" s="41" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="L17" s="45"/>
       <x:c r="M17" s="41" t="str">
@@ -2048,22 +2050,20 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W17" s="41" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="X17" s="41" t="str">
         <x:v>unverified</x:v>
       </x:c>
-      <x:c r="Y17" s="41" t="str">
-        <x:v>YDEX</x:v>
-      </x:c>
+      <x:c r="Y17" s="41" t="str"/>
       <x:c r="Z17" s="41" t="str">
-        <x:v>Финам</x:v>
+        <x:v>Интерфакс</x:v>
       </x:c>
       <x:c r="AA17" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOSmlOMWRURDFvUlZqYktKazJXOFhWR1ZMamNuTGF2QlJ0YmIxTmF6RDMtSHF1Y2RTRkc5QWlnZXQ3WUdUMTB4QUNzUy0zT3I2eGJZSW1DWUxaVDlvR1lrNVhZZ3kybDNrb0tXd0FqMkxHQXNWRFhjcFp0MUI3alRKN1BWdlBSN2V2VWphOUxBQkNjc0l1UDF4WTRKZXkxNHlzSmhIRkhmR2pXc1pKLVV4MzJIN0pLZlVkQ3JvZ2d4aFphcXJkd0F3Z1VKYmdPUUdJ?oc=5</x:v>
+        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE1YcWRJT1pJS3JQYUlDcVBxQmRrd2JFXzdidEJQMkRoTFVIRlBDUnQ5ZjNSMFZGamhRQ1hoTXFwaUVQMW1PZldFWWhvSzdOdmtSQnfSAUtBVV95cUxQWkQ5UHd5NFJieHBKUTVCZURpX1dEWmM4a2FnOXJ3aUREYi04ZGFUclFMNUxBdU1EMFVYWUU4MlhCaXJfTy1NZlVNXzg?oc=5</x:v>
       </x:c>
       <x:c r="AB17" s="41" t="str">
-        <x:v>«Яндекс» вновь выходит на долговой рынок: разбор двойного размещения облигаций - Финам</x:v>
+        <x:v>"Норникель" зафиксировал объем размещения облигаций на уровне 3 млрд юаней - Интерфакс</x:v>
       </x:c>
       <x:c r="AC17" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2071,22 +2071,22 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="41" t="str">
-        <x:v>DL-c0e4b0469b5eb473</x:v>
+        <x:v>DL-f71ff729dc9f5af4</x:v>
       </x:c>
       <x:c r="B18" s="43" t="n">
-        <x:v>46177</x:v>
+        <x:v>46181</x:v>
       </x:c>
       <x:c r="C18" s="41" t="str">
-        <x:v>M&amp;A</x:v>
+        <x:v>DCM</x:v>
       </x:c>
       <x:c r="D18" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E18" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Yandex</x:v>
       </x:c>
       <x:c r="F18" s="41" t="str">
-        <x:v>Ozon</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G18" s="41" t="str">
         <x:v>Not classified</x:v>
@@ -2101,7 +2101,7 @@
       </x:c>
       <x:c r="L18" s="45"/>
       <x:c r="M18" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="N18" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2121,7 +2121,7 @@
         <x:f>IFERROR(IF(AND($J18&gt;0,$P18&gt;0,$K18=$R18),$J18/$P18,""),"")</x:f>
       </x:c>
       <x:c r="U18" s="41" t="str">
-        <x:v>Acquisition / disposal</x:v>
+        <x:v>Bonds</x:v>
       </x:c>
       <x:c r="V18" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2133,16 +2133,16 @@
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y18" s="41" t="str">
-        <x:v>OZON</x:v>
+        <x:v>YDEX</x:v>
       </x:c>
       <x:c r="Z18" s="41" t="str">
-        <x:v>БКС Экспресс</x:v>
+        <x:v>Финам</x:v>
       </x:c>
       <x:c r="AA18" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMioAFBVV95cUxQM0RKYTRnLW8xX0tVdnh1S3RBQ25IUTNrRGtWSTRudTJVU3A3UXpmZjZCR2ItX2NQNmN1aXdPYUpDN0paWHBfUjBNd2xrWWl6Mk9Zel9MREpqcXl1RUpoUXB2MWNPdFBoYV94Mm0zNkVtcVZFM050R2Jqc2ZKQVdlbkVhVmhuNXZpQWd5STAzOW9fYndtQTBpM0JLTWJmMjlq?oc=5</x:v>
+        <x:v>https://www.finam.ru/publications/item/yandeks-vnov-vykhodit-na-dolgovoy-rynok-razbor-dvoynogo-razmeshcheniya-obligatsiy-20260608-1729/</x:v>
       </x:c>
       <x:c r="AB18" s="41" t="str">
-        <x:v>Греф опроверг договоренность Сбера о покупке доли в Озоне - БКС Экспресс</x:v>
+        <x:v>«Яндекс» вновь выходит на долговой рынок: разбор двойного размещения облигаций - Финам</x:v>
       </x:c>
       <x:c r="AC18" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2150,25 +2150,25 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="41" t="str">
-        <x:v>DL-2e27ebc506e38656</x:v>
+        <x:v>DL-c0e4b0469b5eb473</x:v>
       </x:c>
       <x:c r="B19" s="43" t="n">
-        <x:v>46176</x:v>
+        <x:v>46177</x:v>
       </x:c>
       <x:c r="C19" s="41" t="str">
         <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D19" s="41" t="str">
-        <x:v>Completed</x:v>
+        <x:v>Reported</x:v>
       </x:c>
       <x:c r="E19" s="41" t="str">
-        <x:v>Авто.ру</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F19" s="41" t="str">
-        <x:v>Т-Технологии</x:v>
+        <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G19" s="41" t="str">
-        <x:v>Technology</x:v>
+        <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H19" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2206,22 +2206,22 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W19" s="41" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X19" s="41" t="str">
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y19" s="41" t="str">
-        <x:v>YDEX</x:v>
+        <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z19" s="41" t="str">
         <x:v>БКС Экспресс</x:v>
       </x:c>
       <x:c r="AA19" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiowFBVV95cUxNQ0ZvSEhWU1BqUzkyWi1YOWNOR0lab1kxRldxMFV5YllQQWp4Y0xFcjNLTXpHMUFJcnhicWI2RGNuUWRpUndBS0ZlQ2U0c05yWDlTeWZnWG05QjhZR0VWVW5IV19aSkdwa0d1UWpMWC1tLWdicjNtUVk4M2QtbFhsQkFxejdjZ2lLNDYxWTlwUWwyMzhqZ20zelY5SkZpZjBjYzZv?oc=5</x:v>
+        <x:v>https://bcs-express.ru/novosti-i-analitika/gref-oproverg-dogovorennost-sbera-o-pokupke-doli-v-ozone</x:v>
       </x:c>
       <x:c r="AB19" s="41" t="str">
-        <x:v>Т-Технологии закрыли сделку по покупке Авто.ру у Яндекса - БКС Экспресс</x:v>
+        <x:v>Греф опроверг договоренность Сбера о покупке доли в Озоне - БКС Экспресс</x:v>
       </x:c>
       <x:c r="AC19" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2229,10 +2229,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="41" t="str">
-        <x:v>DL-360af9a222272dcf</x:v>
+        <x:v>DL-2e27ebc506e38656</x:v>
       </x:c>
       <x:c r="B20" s="43" t="n">
-        <x:v>46175</x:v>
+        <x:v>46176</x:v>
       </x:c>
       <x:c r="C20" s="41" t="str">
         <x:v>M&amp;A</x:v>
@@ -2241,10 +2241,10 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="E20" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Авто.ру</x:v>
       </x:c>
       <x:c r="F20" s="41" t="str">
-        <x:v>Yandex</x:v>
+        <x:v>Т-Технологии</x:v>
       </x:c>
       <x:c r="G20" s="41" t="str">
         <x:v>Technology</x:v>
@@ -2282,25 +2282,25 @@
         <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V20" s="41" t="str">
-        <x:v>частных инвесторов Яндекса содержит информацию про бизнесы и технологии компании, а также географию присутствия, финансовые результаты, важные новости и многое другое о компании и её рынках</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W20" s="41" t="n">
-        <x:v>9</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="X20" s="41" t="str">
-        <x:v>confirmed</x:v>
+        <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y20" s="41" t="str">
         <x:v>YDEX</x:v>
       </x:c>
       <x:c r="Z20" s="41" t="str">
-        <x:v>Yandex Investor Relations</x:v>
+        <x:v>БКС Экспресс</x:v>
       </x:c>
       <x:c r="AA20" s="41" t="str">
-        <x:v>https://ir.yandex.ru/press-releases?year=2026&amp;id=02-06-2026-04</x:v>
+        <x:v>https://bcs-express.ru/novosti-i-analitika/t-tekhnologii-zakryli-sdelku-po-pokupke-avto-ru-u-iandeksa</x:v>
       </x:c>
       <x:c r="AB20" s="41" t="str">
-        <x:v>Яндекс закрыл сделку по продаже Авто.ру</x:v>
+        <x:v>Т-Технологии закрыли сделку по покупке Авто.ру у Яндекса - БКС Экспресс</x:v>
       </x:c>
       <x:c r="AC20" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2308,7 +2308,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="41" t="str">
-        <x:v>DL-a78cf0af94927306</x:v>
+        <x:v>DL-5eba3b27a4e84dd3</x:v>
       </x:c>
       <x:c r="B21" s="43" t="n">
         <x:v>46175</x:v>
@@ -2317,7 +2317,7 @@
         <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D21" s="41" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E21" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2329,14 +2329,12 @@
         <x:v>Technology</x:v>
       </x:c>
       <x:c r="H21" s="41" t="str">
-        <x:v>Russia</x:v>
-      </x:c>
-      <x:c r="I21" s="44" t="n">
-        <x:v>35000000000</x:v>
-      </x:c>
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I21" s="44"/>
       <x:c r="J21" s="44"/>
       <x:c r="K21" s="41" t="str">
-        <x:v>RUB</x:v>
+        <x:v>NOT DISCLOSED</x:v>
       </x:c>
       <x:c r="L21" s="45"/>
       <x:c r="M21" s="41" t="str">
@@ -2363,25 +2361,25 @@
         <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V21" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>частных инвесторов Яндекса содержит информацию про бизнесы и технологии компании, а также географию присутствия, финансовые результаты, важные новости и многое другое о компании и её рынках</x:v>
       </x:c>
       <x:c r="W21" s="41" t="n">
-        <x:v>4</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="X21" s="41" t="str">
-        <x:v>unverified</x:v>
+        <x:v>confirmed</x:v>
       </x:c>
       <x:c r="Y21" s="41" t="str">
         <x:v>YDEX</x:v>
       </x:c>
       <x:c r="Z21" s="41" t="str">
-        <x:v>Финам</x:v>
+        <x:v>Yandex Investor Relations</x:v>
       </x:c>
       <x:c r="AA21" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMilgFBVV95cUxQWFk5YjhpaHc0S3BiTEpUVzFndHdkTDVmY0EtRDhFQ0pYcjBvWUF3V3FZUFhaUjhEQ1FXT0FDdWU1dGdtVmJ1Z1l5bmhGcVBwdjhsWTZVNG10dWhmTlNGbGZqV2cwRUoyaEdZS3c0dEx1MV8ySGpfX2ljQnhfemFELThnSDc3T09JZ1lOZW45Yk93YmYyb3c?oc=5</x:v>
+        <x:v>https://ir.yandex.ru/press-releases?year=2026&amp;id=02-06-2026-04</x:v>
       </x:c>
       <x:c r="AB21" s="41" t="str">
-        <x:v>"Яндекс" продал "Авто.ру" "Т-Технологиям" за 35 млрд рублей - Финам</x:v>
+        <x:v>Яндекс закрыл сделку по продаже Авто.ру</x:v>
       </x:c>
       <x:c r="AC21" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2389,10 +2387,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="41" t="str">
-        <x:v>DL-a4f6a4524ddca358</x:v>
+        <x:v>DL-a78cf0af94927306</x:v>
       </x:c>
       <x:c r="B22" s="43" t="n">
-        <x:v>46170</x:v>
+        <x:v>46175</x:v>
       </x:c>
       <x:c r="C22" s="41" t="str">
         <x:v>M&amp;A</x:v>
@@ -2404,18 +2402,20 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F22" s="41" t="str">
-        <x:v>Ozon</x:v>
+        <x:v>Yandex</x:v>
       </x:c>
       <x:c r="G22" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Technology</x:v>
       </x:c>
       <x:c r="H22" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
-      <x:c r="I22" s="44"/>
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I22" s="44" t="n">
+        <x:v>35000000000</x:v>
+      </x:c>
       <x:c r="J22" s="44"/>
       <x:c r="K22" s="41" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="L22" s="45"/>
       <x:c r="M22" s="41" t="str">
@@ -2445,22 +2445,22 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W22" s="41" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X22" s="41" t="str">
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y22" s="41" t="str">
-        <x:v>OZON</x:v>
+        <x:v>YDEX</x:v>
       </x:c>
       <x:c r="Z22" s="41" t="str">
-        <x:v>Интерфакс</x:v>
+        <x:v>Финам</x:v>
       </x:c>
       <x:c r="AA22" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE9GMUxsS2ZKR2JaU2ZhY1hRSmoteVVNM1V6U2pJQnFGblRETXk1b0pLLXl3VXNvREgwdVg4dmNyc3VBVWxFZ1ZjUmxILXlrWU80VVHSAUtBVV95cUxPM21YSmF3aGRJQThYblp1MEEyNGNLSnR0SzlnTG1ITWtJWXY5bU1Jdm9kWU5nRjRYOUoxRlFscTB5X2NHVUlWYmtDX0k?oc=5</x:v>
+        <x:v>https://www.finam.ru/publications/item/yandeks-prodal-avtoru-t-tekhnologiyam-20260602-1802/</x:v>
       </x:c>
       <x:c r="AB22" s="41" t="str">
-        <x:v>"Ъ" сообщил о переговорах структур Сбера с АФК "Система" о покупке доли в Ozon - Интерфакс</x:v>
+        <x:v>"Яндекс" продал "Авто.ру" "Т-Технологиям" за 35 млрд рублей - Финам</x:v>
       </x:c>
       <x:c r="AC22" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2468,33 +2468,35 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="41" t="str">
-        <x:v>DL-e08040bba3b952c1</x:v>
+        <x:v>DL-1f4ea43fab1ad3e7</x:v>
       </x:c>
       <x:c r="B23" s="43" t="n">
-        <x:v>46170</x:v>
+        <x:v>46171</x:v>
       </x:c>
       <x:c r="C23" s="41" t="str">
         <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D23" s="41" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Potential</x:v>
       </x:c>
       <x:c r="E23" s="41" t="str">
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F23" s="41" t="str">
-        <x:v>Yandex</x:v>
+        <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G23" s="41" t="str">
         <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H23" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
-      <x:c r="I23" s="44"/>
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I23" s="44" t="n">
+        <x:v>300000000000</x:v>
+      </x:c>
       <x:c r="J23" s="44"/>
       <x:c r="K23" s="41" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="L23" s="45"/>
       <x:c r="M23" s="41" t="str">
@@ -2530,16 +2532,16 @@
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y23" s="41" t="str">
-        <x:v>YDEX</x:v>
+        <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z23" s="41" t="str">
-        <x:v>Финам</x:v>
+        <x:v>Сибирское информационное агентство</x:v>
       </x:c>
       <x:c r="AA23" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMirAFBVV95cUxNSlk2WU9xYjNqM1AwRkNGOV9BYnhzQVg3VlRaaWJlT01VVDNrYklwUjY4SFZfdjZQLVlHZEpxYm0tVmpDUFN5a190bUU0MnFnb2VFMFMyQ2E1OWlyQ2djRWwtdWMyN3F5NXRYamZkUmFhMkk4UlFZQXFDOVB2RE9uNjZkdFFMbGZFT0dWOTN4MjZDbXZmMzNSOUNlOXVaZjJGcmM4QnZiM0I3QUhM?oc=5</x:v>
+        <x:v>https://sia.ru/?section\=484\&amp;action\=show_news\&amp;id\=16828609</x:v>
       </x:c>
       <x:c r="AB23" s="41" t="str">
-        <x:v>"Яндекс" стал основным претендентом на покупку "Островка" - Финам</x:v>
+        <x:v>«Сбер» может стать совладельцем Ozon в сделке на 300 млрд рублей? - Сибирское информационное агентство</x:v>
       </x:c>
       <x:c r="AC23" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2547,7 +2549,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="41" t="str">
-        <x:v>DL-4ffd21b67b0042b7</x:v>
+        <x:v>DL-a4f6a4524ddca358</x:v>
       </x:c>
       <x:c r="B24" s="43" t="n">
         <x:v>46170</x:v>
@@ -2556,7 +2558,7 @@
         <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D24" s="41" t="str">
-        <x:v>Potential</x:v>
+        <x:v>Reported</x:v>
       </x:c>
       <x:c r="E24" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2568,14 +2570,12 @@
         <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H24" s="41" t="str">
-        <x:v>Russia</x:v>
-      </x:c>
-      <x:c r="I24" s="44" t="n">
-        <x:v>30000000000</x:v>
-      </x:c>
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I24" s="44"/>
       <x:c r="J24" s="44"/>
       <x:c r="K24" s="41" t="str">
-        <x:v>RUB</x:v>
+        <x:v>NOT DISCLOSED</x:v>
       </x:c>
       <x:c r="L24" s="45"/>
       <x:c r="M24" s="41" t="str">
@@ -2605,7 +2605,7 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W24" s="41" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="X24" s="41" t="str">
         <x:v>unverified</x:v>
@@ -2614,13 +2614,13 @@
         <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z24" s="41" t="str">
-        <x:v>RB.ru</x:v>
+        <x:v>Интерфакс</x:v>
       </x:c>
       <x:c r="AA24" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMixAFBVV95cUxOZGNTQll0aVZOSDFubmt0bU5BdWNXNVA0WFZaOFdKa3B1VkctYXdkU25tLVdQSlNjNjFBYzA0ZzFYbVZKRnNKMk9Cb3RkSFYtaVFUR0JVc0pMNkNFUnFaeUdJX1JKRWlqMUZKeHo3UTZNaDU3LUc2RWxDd2FMYTUyUTEtY1dhcHFUVlJ4ZDlDS19SVkF5a0tqS0duRkljSWNNN0NLajJrSDZVdDNNR2ZfNVlyTVBvb0xFOXdFYmtpb2ZjTXRi?oc=5</x:v>
+        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE9GMUxsS2ZKR2JaU2ZhY1hRSmoteVVNM1V6U2pJQnFGblRETXk1b0pLLXl3VXNvREgwdVg4dmNyc3VBVWxFZ1ZjUmxILXlrWU80VVHSAUtBVV95cUxPM21YSmF3aGRJQThYblp1MEEyNGNLSnR0SzlnTG1ITWtJWXY5bU1Jdm9kWU5nRjRYOUoxRlFscTB5X2NHVUlWYmtDX0k?oc=5</x:v>
       </x:c>
       <x:c r="AB24" s="41" t="str">
-        <x:v>Сбер может купить долю инвесткомпании АФК «Система» в Ozon за 30 млрд рублей - RB.ru</x:v>
+        <x:v>"Ъ" сообщил о переговорах структур Сбера с АФК "Система" о покупке доли в Ozon - Интерфакс</x:v>
       </x:c>
       <x:c r="AC24" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2628,7 +2628,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="41" t="str">
-        <x:v>DL-ca53a880a58471a3</x:v>
+        <x:v>DL-e08040bba3b952c1</x:v>
       </x:c>
       <x:c r="B25" s="43" t="n">
         <x:v>46170</x:v>
@@ -2643,10 +2643,10 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F25" s="41" t="str">
-        <x:v>Ozon</x:v>
+        <x:v>Yandex</x:v>
       </x:c>
       <x:c r="G25" s="41" t="str">
-        <x:v>Financials</x:v>
+        <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H25" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2690,16 +2690,16 @@
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y25" s="41" t="str">
-        <x:v>OZON</x:v>
+        <x:v>YDEX</x:v>
       </x:c>
       <x:c r="Z25" s="41" t="str">
-        <x:v>Альфа-Банк</x:v>
+        <x:v>Финам</x:v>
       </x:c>
       <x:c r="AA25" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMihgFBVV95cUxOVVc5b2xRd2dWREJQMEVGcEVKSlhNdFFmTjNGYWVnRkRNbHlmZ29zRGdzUjlrS2VQQjJxM0RhUTh4bnhIWnhNb3ZnQ2VhYmJqdEI1Q0dpVHZOWlNCLXNUanVlYTdhNmQ2TkpGZ1hFVG0xclRWNWZvZUhmeXdua1BtUDNpMm9LZw?oc=5</x:v>
+        <x:v>https://www.finam.ru/publications/item/yandeks-stal-osnovnym-pretendentom-na-pokupku-ostrovka-20260528-0928/</x:v>
       </x:c>
       <x:c r="AB25" s="41" t="str">
-        <x:v>Сбер забирает Ozon. Инсайд или вброс? Кто выиграет от сделки? - Альфа-Банк</x:v>
+        <x:v>"Яндекс" стал основным претендентом на покупку "Островка" - Финам</x:v>
       </x:c>
       <x:c r="AC25" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2707,7 +2707,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="41" t="str">
-        <x:v>DL-eee2cc5f0b30c3ba</x:v>
+        <x:v>DL-4ffd21b67b0042b7</x:v>
       </x:c>
       <x:c r="B26" s="43" t="n">
         <x:v>46170</x:v>
@@ -2716,7 +2716,7 @@
         <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D26" s="41" t="str">
-        <x:v>Reported</x:v>
+        <x:v>Potential</x:v>
       </x:c>
       <x:c r="E26" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2725,15 +2725,17 @@
         <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G26" s="41" t="str">
-        <x:v>Financials</x:v>
+        <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H26" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
-      <x:c r="I26" s="44"/>
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I26" s="44" t="n">
+        <x:v>30000000000</x:v>
+      </x:c>
       <x:c r="J26" s="44"/>
       <x:c r="K26" s="41" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="L26" s="45"/>
       <x:c r="M26" s="41" t="str">
@@ -2772,13 +2774,13 @@
         <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z26" s="41" t="str">
-        <x:v>Альфа-Банк</x:v>
+        <x:v>RB.ru</x:v>
       </x:c>
       <x:c r="AA26" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMihgFBVV95cUxPa1Utd0tlY3RsT1JNSUZEcGdEdG84bFBJYlc0eDVEand3UnppVTduOUZPMUo2UHJ6SmxSSGgwekt6cDFyS3ByZDRxR1RrQjNJWk5VUlB4U2UyM0pSa3FiNnRscllQT19fZ2pEb0xQTU4xdXNXTi1PbWxNTF9LRTg2RTh3VHoyZw?oc=5</x:v>
+        <x:v>https://rb.ru/news/sber-mozhet-kupit-akcii-v-ozon-na-30-mlrd-investkompaniya-afk-sistema-otricaet-informaciyu-o-prodazhe-doli/</x:v>
       </x:c>
       <x:c r="AB26" s="41" t="str">
-        <x:v>Озон и Сбер, сделки не будет? - Альфа-Банк</x:v>
+        <x:v>Сбер может купить долю инвесткомпании АФК «Система» в Ozon за 30 млрд рублей - RB.ru</x:v>
       </x:c>
       <x:c r="AC26" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2786,10 +2788,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="41" t="str">
-        <x:v>DL-54c26c1e05d520bd</x:v>
+        <x:v>DL-ca53a880a58471a3</x:v>
       </x:c>
       <x:c r="B27" s="43" t="n">
-        <x:v>46167</x:v>
+        <x:v>46170</x:v>
       </x:c>
       <x:c r="C27" s="41" t="str">
         <x:v>M&amp;A</x:v>
@@ -2804,7 +2806,7 @@
         <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G27" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Financials</x:v>
       </x:c>
       <x:c r="H27" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2816,7 +2818,7 @@
       </x:c>
       <x:c r="L27" s="45"/>
       <x:c r="M27" s="41" t="str">
-        <x:v>Shares</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="N27" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2851,13 +2853,13 @@
         <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z27" s="41" t="str">
-        <x:v>Финам</x:v>
+        <x:v>Альфа-Банк</x:v>
       </x:c>
       <x:c r="AA27" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMirwFBVV95cUxNckFiOGoyLVd2REpiUVVDaWp6NzF5Y1laekdUZnhnWUJYS3ZteHpxSGd6OElyTUwyZXVFWjgwWmRFclVXbV9FR2xKS2dHZDdoZEZsUEMycy01ZUxUMU03eTBybC1NQlZ5dDVtZHp4NTdVdEhzak9jVlgwZ2ZXTVA0SnIyM0RUTG5saEdQWG5FTDIwUmE1MHllN2xOek1HeXlRS2RtSDhCeFZfaElpRy1F?oc=5</x:v>
+        <x:v>https://alfabank.ru/alfa-investor/posts/t/2af58b47-265b-f111-91c6-0050569e1fd0/</x:v>
       </x:c>
       <x:c r="AB27" s="41" t="str">
-        <x:v>25.05.26 Последний день покупки акций “Озона” под дивиденды - 25 мая - Финам</x:v>
+        <x:v>Сбер забирает Ozon. Инсайд или вброс? Кто выиграет от сделки? - Альфа-Банк</x:v>
       </x:c>
       <x:c r="AC27" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2865,22 +2867,22 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="41" t="str">
-        <x:v>DL-38b5154e2b53df8c</x:v>
+        <x:v>DL-eee2cc5f0b30c3ba</x:v>
       </x:c>
       <x:c r="B28" s="43" t="n">
-        <x:v>46157</x:v>
+        <x:v>46170</x:v>
       </x:c>
       <x:c r="C28" s="41" t="str">
-        <x:v>ECM</x:v>
+        <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D28" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E28" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="F28" s="41" t="str">
         <x:v>Ozon</x:v>
-      </x:c>
-      <x:c r="F28" s="41" t="str">
-        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G28" s="41" t="str">
         <x:v>Financials</x:v>
@@ -2895,7 +2897,7 @@
       </x:c>
       <x:c r="L28" s="45"/>
       <x:c r="M28" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="N28" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2915,7 +2917,7 @@
         <x:f>IFERROR(IF(AND($J28&gt;0,$P28&gt;0,$K28=$R28),$J28/$P28,""),"")</x:f>
       </x:c>
       <x:c r="U28" s="41" t="str">
-        <x:v>Equity issuance</x:v>
+        <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V28" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -2930,13 +2932,13 @@
         <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z28" s="41" t="str">
-        <x:v>Финам</x:v>
+        <x:v>Альфа-Банк</x:v>
       </x:c>
       <x:c r="AA28" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMi7gFBVV95cUxOVkF3VWdna082MXVoUDVVTnpvUjV1Y2tnMGRwRkYwRlhnUE1RZldyUGVCcklzSWdXQmhMYkRaNi1nZGp5LVdzU3RRWV9kTnpJbFFxU2lCSGR1clk5R3NIaDZHeDRxTUF6VkZHV2F4dTAtS0Jjd1FEM281dU5YZ3lMRWROOVNiT29mVG1EcXRCcmdmaDZ5OFpzTmRHRWpidFMzdjktZHhRMGpxZ0pUZmw0MDRGNjZEMWFPVC1EcFFFa1NFNzJlNk1oUnI1cGFpc2ZDYWk0LUxuaVN1LUdvU25hTXpINjhQZGNHdzJIdElR?oc=5</x:v>
+        <x:v>https://alfabank.ru/alfa-investor/posts/t/06d3da91-dd5a-f111-91c6-0050569e1fd0/</x:v>
       </x:c>
       <x:c r="AB28" s="41" t="str">
-        <x:v>Отчетности «Займера», БСП и «Совкомбанка», дивидендный вопрос у «Озона» и «МД Медикал» - основные события 15 мая 15.05.2026 - Финам</x:v>
+        <x:v>Озон и Сбер, сделки не будет? - Альфа-Банк</x:v>
       </x:c>
       <x:c r="AC28" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -2944,10 +2946,10 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="41" t="str">
-        <x:v>DL-32f044efd41bc454</x:v>
+        <x:v>DL-4d23d3c416f43c48</x:v>
       </x:c>
       <x:c r="B29" s="43" t="n">
-        <x:v>46157</x:v>
+        <x:v>46170</x:v>
       </x:c>
       <x:c r="C29" s="41" t="str">
         <x:v>M&amp;A</x:v>
@@ -2959,7 +2961,7 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F29" s="41" t="str">
-        <x:v>VKCO</x:v>
+        <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G29" s="41" t="str">
         <x:v>Not classified</x:v>
@@ -2972,7 +2974,9 @@
       <x:c r="K29" s="41" t="str">
         <x:v>NOT DISCLOSED</x:v>
       </x:c>
-      <x:c r="L29" s="45"/>
+      <x:c r="L29" s="45" t="n">
+        <x:v>0.07</x:v>
+      </x:c>
       <x:c r="M29" s="41" t="str">
         <x:v>Shares</x:v>
       </x:c>
@@ -3000,20 +3004,22 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W29" s="41" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X29" s="41" t="str">
         <x:v>unverified</x:v>
       </x:c>
-      <x:c r="Y29" s="41" t="str"/>
+      <x:c r="Y29" s="41" t="str">
+        <x:v>OZON</x:v>
+      </x:c>
       <x:c r="Z29" s="41" t="str">
-        <x:v>Интерфакс</x:v>
+        <x:v>Финам</x:v>
       </x:c>
       <x:c r="AA29" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE1SRWp6YUhObThSanNWWnBCQjlnX0xPVW1fQzJPSlJxM3JxcVhVTWlJaWZVcW5VNXFTQjU0RkJ6cC0wem9DTUNLZWlXeXZmMDhyUlHSAUtBVV95cUxPaFhNLWM1eThHQVJpOEg0TEpxT1BjRk5IdTEyYmFOdzNCOEluQmtLU3pmcXViOW5PM1gwR3ZsT2RhZEVCLTkwQ1RMZk0?oc=5</x:v>
+        <x:v>https://www.finam.ru/publications/item/aktsii-afk-sistema-podskochili-na-7-na-soobshcheniyakh-o-pokupke-doli-ozona-strukturami-sbera-20260528-1910/</x:v>
       </x:c>
       <x:c r="AB29" s="41" t="str">
-        <x:v>Трамп в I квартале совершал сделки с акциями Nvidia и Boeing - Интерфакс</x:v>
+        <x:v>Акции АФК "Система" подскочили на 7% на сообщениях о покупке доли "Озона" структурами "Сбера" - Финам</x:v>
       </x:c>
       <x:c r="AC29" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3021,39 +3027,37 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="41" t="str">
-        <x:v>DL-71608263fecb5e53</x:v>
+        <x:v>DL-54c26c1e05d520bd</x:v>
       </x:c>
       <x:c r="B30" s="43" t="n">
-        <x:v>46150</x:v>
+        <x:v>46167</x:v>
       </x:c>
       <x:c r="C30" s="41" t="str">
-        <x:v>DCM</x:v>
+        <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D30" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E30" s="41" t="str">
-        <x:v>Делимобиль</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F30" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G30" s="41" t="str">
         <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H30" s="41" t="str">
-        <x:v>Russia</x:v>
-      </x:c>
-      <x:c r="I30" s="44" t="n">
-        <x:v>1900000000</x:v>
-      </x:c>
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I30" s="44"/>
       <x:c r="J30" s="44"/>
       <x:c r="K30" s="41" t="str">
-        <x:v>RUB</x:v>
+        <x:v>NOT DISCLOSED</x:v>
       </x:c>
       <x:c r="L30" s="45"/>
       <x:c r="M30" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>Shares</x:v>
       </x:c>
       <x:c r="N30" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3073,26 +3077,28 @@
         <x:f>IFERROR(IF(AND($J30&gt;0,$P30&gt;0,$K30=$R30),$J30/$P30,""),"")</x:f>
       </x:c>
       <x:c r="U30" s="41" t="str">
-        <x:v>Bonds</x:v>
+        <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V30" s="41" t="str">
-        <x:v>погашения выпуска облигаций на 1,9 млрд рублей</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W30" s="41" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X30" s="41" t="str">
         <x:v>unverified</x:v>
       </x:c>
-      <x:c r="Y30" s="41" t="str"/>
+      <x:c r="Y30" s="41" t="str">
+        <x:v>OZON</x:v>
+      </x:c>
       <x:c r="Z30" s="41" t="str">
-        <x:v>Интерфакс</x:v>
+        <x:v>Финам</x:v>
       </x:c>
       <x:c r="AA30" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE5rRHd6NXMzNkpDcVZDdVR4NXhZN185LXRRSDMzVzZiUGd4cmNqV1BydzRLTnh4cHJnU19qNnQ1X05XMDl6VnBjVlBXY0NUOUZ3VlHSAUtBVV95cUxQOHVvOS00aURkZ3lDUGZ6Sk9kYTVFSDJhcGNJQk1PVVR2ZFJwWnZlRGZ4eW85TS15QUs4bmkxOWUzQW5PbGpDeUVnOVk?oc=5</x:v>
+        <x:v>https://www.finam.ru/publications/item/posledniy-den-pokupki-aktsiy-ozona-pod-dividendy-25-maya-20260525-0652/</x:v>
       </x:c>
       <x:c r="AB30" s="41" t="str">
-        <x:v>"Делимобиль" перечислил в НРД средства для погашения выпуска облигаций на 1,9 млрд рублей - Интерфакс</x:v>
+        <x:v>25.05.26 Последний день покупки акций “Озона” под дивиденды - 25 мая - Финам</x:v>
       </x:c>
       <x:c r="AC30" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3100,10 +3106,10 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="41" t="str">
-        <x:v>DL-2848bdd8b067faa2</x:v>
+        <x:v>DL-38b5154e2b53df8c</x:v>
       </x:c>
       <x:c r="B31" s="43" t="n">
-        <x:v>46147</x:v>
+        <x:v>46157</x:v>
       </x:c>
       <x:c r="C31" s="41" t="str">
         <x:v>ECM</x:v>
@@ -3112,23 +3118,21 @@
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E31" s="41" t="str">
-        <x:v>Yandex</x:v>
+        <x:v>Ozon</x:v>
       </x:c>
       <x:c r="F31" s="41" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G31" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Financials</x:v>
       </x:c>
       <x:c r="H31" s="41" t="str">
-        <x:v>Russia</x:v>
-      </x:c>
-      <x:c r="I31" s="44" t="n">
-        <x:v>50000000000</x:v>
-      </x:c>
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I31" s="44"/>
       <x:c r="J31" s="44"/>
       <x:c r="K31" s="41" t="str">
-        <x:v>RUB</x:v>
+        <x:v>NOT DISCLOSED</x:v>
       </x:c>
       <x:c r="L31" s="45"/>
       <x:c r="M31" s="41" t="str">
@@ -3164,16 +3168,16 @@
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y31" s="41" t="str">
-        <x:v>YDEX</x:v>
+        <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z31" s="41" t="str">
-        <x:v>БКС Экспресс</x:v>
+        <x:v>Финам</x:v>
       </x:c>
       <x:c r="AA31" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMikwFBVV95cUxPbkRNMVpoTFN4cXlrOWRya3A4SW1Dd09IUHIzMUw3emMzY1hZckpPRWtMclI2aTllZTRQTlRwUmNGNVp4X1hPV041elJSWGhtVS1kM0VGMFpWdmZIcDRmTS04MjBSb3FoVG5xZWdhY0REZkxLMTMxTE1PeF92VW5SRkxDYVNrVGVuNVFTSlRfaFFFeWc?oc=5</x:v>
+        <x:v>https://www.finam.ru/publications/item/otchetnosti-zaymera-bsp-i-sovkombanka-dividendnyy-vopros-u-ozona-i-md-medikal-osnovnye-sobytiya-15-maya-20260515-0900/</x:v>
       </x:c>
       <x:c r="AB31" s="41" t="str">
-        <x:v>Яндекс одобрил выкуп акций на 50 млрд рублей - БКС Экспресс</x:v>
+        <x:v>Отчетности «Займера», БСП и «Совкомбанка», дивидендный вопрос у «Озона» и «МД Медикал» - основные события 15 мая 15.05.2026 - Финам</x:v>
       </x:c>
       <x:c r="AC31" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3181,25 +3185,25 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="41" t="str">
-        <x:v>DL-3d4a31cc3b7936d0</x:v>
+        <x:v>DL-32f044efd41bc454</x:v>
       </x:c>
       <x:c r="B32" s="43" t="n">
-        <x:v>46146</x:v>
+        <x:v>46157</x:v>
       </x:c>
       <x:c r="C32" s="41" t="str">
-        <x:v>ECM</x:v>
+        <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D32" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E32" s="41" t="str">
-        <x:v>Yandex</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F32" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>VKCO</x:v>
       </x:c>
       <x:c r="G32" s="41" t="str">
-        <x:v>Energy</x:v>
+        <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H32" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3211,7 +3215,7 @@
       </x:c>
       <x:c r="L32" s="45"/>
       <x:c r="M32" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>Shares</x:v>
       </x:c>
       <x:c r="N32" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3231,28 +3235,26 @@
         <x:f>IFERROR(IF(AND($J32&gt;0,$P32&gt;0,$K32=$R32),$J32/$P32,""),"")</x:f>
       </x:c>
       <x:c r="U32" s="41" t="str">
-        <x:v>Equity issuance</x:v>
+        <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V32" s="41" t="str">
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W32" s="41" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="X32" s="41" t="str">
         <x:v>unverified</x:v>
       </x:c>
-      <x:c r="Y32" s="41" t="str">
-        <x:v>YDEX, OZON</x:v>
-      </x:c>
+      <x:c r="Y32" s="41" t="str"/>
       <x:c r="Z32" s="41" t="str">
-        <x:v>SberCIB</x:v>
+        <x:v>Интерфакс</x:v>
       </x:c>
       <x:c r="AA32" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQZEltanhoOVlVS2FSRnNObHRXRkJnUEpjZ1VRXzB4czdNUFJOVzVxNU1XcGdxX1gxNmhYcHVrWFh1bXZMRTA5UUZHczhJNlJLYl8wVzdtZmdWYjRQZVB4TDVRNHNURVI1UkhkeVFpNXN4WnhUekFURDhiSlFyZDAtUFMtNW1VR3JEZFUwMEktbmFIYk52Uy02ay1IQTdYZHE2Zm10Vkw1LVBLdw?oc=5</x:v>
+        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE1SRWp6YUhObThSanNWWnBCQjlnX0xPVW1fQzJPSlJxM3JxcVhVTWlJaWZVcW5VNXFTQjU0RkJ6cC0wem9DTUNLZWlXeXZmMDhyUlHSAUtBVV95cUxPaFhNLWM1eThHQVJpOEg0TEpxT1BjRk5IdTEyYmFOdzNCOEluQmtLU3pmcXViOW5PM1gwR3ZsT2RhZEVCLTkwQ1RMZk0?oc=5</x:v>
       </x:c>
       <x:c r="AB32" s="41" t="str">
-        <x:v>Результаты Ozon, ДОМ. РФ, дивиденды Яндекса и Татнефти и другие новости недели - SberCIB</x:v>
+        <x:v>Трамп в I квартале совершал сделки с акциями Nvidia и Boeing - Интерфакс</x:v>
       </x:c>
       <x:c r="AC32" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3260,37 +3262,39 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="41" t="str">
-        <x:v>DL-6bc0569f7ac374fe</x:v>
+        <x:v>DL-71608263fecb5e53</x:v>
       </x:c>
       <x:c r="B33" s="43" t="n">
-        <x:v>46139</x:v>
+        <x:v>46150</x:v>
       </x:c>
       <x:c r="C33" s="41" t="str">
-        <x:v>M&amp;A</x:v>
+        <x:v>DCM</x:v>
       </x:c>
       <x:c r="D33" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E33" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Делимобиль</x:v>
       </x:c>
       <x:c r="F33" s="41" t="str">
-        <x:v>Ozon</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G33" s="41" t="str">
-        <x:v>Financials</x:v>
+        <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H33" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
-      <x:c r="I33" s="44"/>
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I33" s="44" t="n">
+        <x:v>1900000000</x:v>
+      </x:c>
       <x:c r="J33" s="44"/>
       <x:c r="K33" s="41" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="L33" s="45"/>
       <x:c r="M33" s="41" t="str">
-        <x:v>Shares</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="N33" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3310,28 +3314,26 @@
         <x:f>IFERROR(IF(AND($J33&gt;0,$P33&gt;0,$K33=$R33),$J33/$P33,""),"")</x:f>
       </x:c>
       <x:c r="U33" s="41" t="str">
-        <x:v>Acquisition / disposal</x:v>
+        <x:v>Bonds</x:v>
       </x:c>
       <x:c r="V33" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>погашения выпуска облигаций на 1,9 млрд рублей</x:v>
       </x:c>
       <x:c r="W33" s="41" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="X33" s="41" t="str">
         <x:v>unverified</x:v>
       </x:c>
-      <x:c r="Y33" s="41" t="str">
-        <x:v>OZON</x:v>
-      </x:c>
+      <x:c r="Y33" s="41" t="str"/>
       <x:c r="Z33" s="41" t="str">
-        <x:v>Ведомости</x:v>
+        <x:v>Интерфакс</x:v>
       </x:c>
       <x:c r="AA33" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMifkFVX3lxTE5wcVN1bk9QeWE3N3kxMkdGdndraERVOGhyUndZcTkwSVVWdlhXUkVldXUtRWR5QTlCR3owOHN1QzFPZVVDR0JWMGkweTM2ekRobml3MzJqT3ZyTGFCSTZtTk0yZ3FxOG52ZjA3c203bEJ4UGVIN18xQUJxenBLQQ?oc=5</x:v>
+        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE5rRHd6NXMzNkpDcVZDdVR4NXhZN185LXRRSDMzVzZiUGd4cmNqV1BydzRLTnh4cHJnU19qNnQ1X05XMDl6VnBjVlBXY0NUOUZ3VlHSAUtBVV95cUxQOHVvOS00aURkZ3lDUGZ6Sk9kYTVFSDJhcGNJQk1PVVR2ZFJwWnZlRGZ4eW85TS15QUs4bmkxOWUzQW5PbGpDeUVnOVk?oc=5</x:v>
       </x:c>
       <x:c r="AB33" s="41" t="str">
-        <x:v>Путин исключил «Озон банк» из списка с запретом на сделки с акциями и долями - Ведомости</x:v>
+        <x:v>"Делимобиль" перечислил в НРД средства для погашения выпуска облигаций на 1,9 млрд рублей - Интерфакс</x:v>
       </x:c>
       <x:c r="AC33" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3339,37 +3341,39 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="41" t="str">
-        <x:v>DL-cc671fa6b14f8f28</x:v>
+        <x:v>DL-2848bdd8b067faa2</x:v>
       </x:c>
       <x:c r="B34" s="43" t="n">
-        <x:v>46139</x:v>
+        <x:v>46147</x:v>
       </x:c>
       <x:c r="C34" s="41" t="str">
-        <x:v>M&amp;A</x:v>
+        <x:v>ECM</x:v>
       </x:c>
       <x:c r="D34" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E34" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Yandex</x:v>
       </x:c>
       <x:c r="F34" s="41" t="str">
-        <x:v>Ozon</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G34" s="41" t="str">
-        <x:v>Financials</x:v>
+        <x:v>Not classified</x:v>
       </x:c>
       <x:c r="H34" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
-      <x:c r="I34" s="44"/>
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I34" s="44" t="n">
+        <x:v>50000000000</x:v>
+      </x:c>
       <x:c r="J34" s="44"/>
       <x:c r="K34" s="41" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="L34" s="45"/>
       <x:c r="M34" s="41" t="str">
-        <x:v>Shares</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="N34" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3389,7 +3393,7 @@
         <x:f>IFERROR(IF(AND($J34&gt;0,$P34&gt;0,$K34=$R34),$J34/$P34,""),"")</x:f>
       </x:c>
       <x:c r="U34" s="41" t="str">
-        <x:v>Acquisition / disposal</x:v>
+        <x:v>Equity issuance</x:v>
       </x:c>
       <x:c r="V34" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3401,16 +3405,16 @@
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y34" s="41" t="str">
-        <x:v>OZON</x:v>
+        <x:v>YDEX</x:v>
       </x:c>
       <x:c r="Z34" s="41" t="str">
         <x:v>БКС Экспресс</x:v>
       </x:c>
       <x:c r="AA34" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiwgFBVV95cUxORlpPNHotYkNzQVpwd2ptLTRIVmJmelQwVHY5Vjc2Rmd1YzFnMW52R3h3aXlFYkpzc0NfY0NPdWk3RnhUSXhudGhZUWxXeE90WlNpVmRkYlhxSlNHLXFkZ1pLMllFY3VBQUx6bDJUcG13VEVINVlKOTFMUkRkUUx0bllTQ2NQdzBaMENTM3FrN2dMNVFjQ2NKRTVUNG92QWlpcEdtWVFuMWx1dnJRTTFWS1paVllydW9oeUU0NjNUVjhCUQ?oc=5</x:v>
+        <x:v>https://bcs-express.ru/novosti-i-analitika/iandeks-odobril-vykup-aktsii-na-50-mlrd-rublei</x:v>
       </x:c>
       <x:c r="AB34" s="41" t="str">
-        <x:v>Ozon Банк исключен из перечня банков, с акциями которых запрещены сделки - БКС Экспресс</x:v>
+        <x:v>Яндекс одобрил выкуп акций на 50 млрд рублей - БКС Экспресс</x:v>
       </x:c>
       <x:c r="AC34" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3418,25 +3422,25 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="41" t="str">
-        <x:v>DL-2d1ef3023240f32a</x:v>
+        <x:v>DL-3d4a31cc3b7936d0</x:v>
       </x:c>
       <x:c r="B35" s="43" t="n">
-        <x:v>46139</x:v>
+        <x:v>46146</x:v>
       </x:c>
       <x:c r="C35" s="41" t="str">
-        <x:v>M&amp;A</x:v>
+        <x:v>ECM</x:v>
       </x:c>
       <x:c r="D35" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E35" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Yandex</x:v>
       </x:c>
       <x:c r="F35" s="41" t="str">
-        <x:v>Ozon</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G35" s="41" t="str">
-        <x:v>Financials</x:v>
+        <x:v>Energy</x:v>
       </x:c>
       <x:c r="H35" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3448,7 +3452,7 @@
       </x:c>
       <x:c r="L35" s="45"/>
       <x:c r="M35" s="41" t="str">
-        <x:v>Shares</x:v>
+        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="N35" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3468,7 +3472,7 @@
         <x:f>IFERROR(IF(AND($J35&gt;0,$P35&gt;0,$K35=$R35),$J35/$P35,""),"")</x:f>
       </x:c>
       <x:c r="U35" s="41" t="str">
-        <x:v>Acquisition / disposal</x:v>
+        <x:v>Equity issuance</x:v>
       </x:c>
       <x:c r="V35" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3480,16 +3484,16 @@
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y35" s="41" t="str">
-        <x:v>OZON</x:v>
+        <x:v>YDEX, OZON</x:v>
       </x:c>
       <x:c r="Z35" s="41" t="str">
-        <x:v>Главпортал</x:v>
+        <x:v>SberCIB</x:v>
       </x:c>
       <x:c r="AA35" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMifEFVX3lxTE5vODZHWnJJX1RoLWU3X2RfSGpCZFZrN2xZeGtyOVVzSENxQzlaQTEwV3pCNXBuOG9JRnVfTkdxOGl5N3RJTGhDVVh0YXdBbTY5dnlZYWRjVkJ5MTFROHhTQUVvdjEwS3BpYUtmSG12YmVocnBnVmVpVmN0ZzQ?oc=5</x:v>
+        <x:v>https://sbercib.ru/publication/rezultati-ozon-dom-rf-dividendi-yandeksa-i-tatnefti-i-drugie-novosti-nedeli</x:v>
       </x:c>
       <x:c r="AB35" s="41" t="str">
-        <x:v>Путин разрешил сделки с акциями «Озон банка» - Главпортал</x:v>
+        <x:v>Результаты Ozon, ДОМ. РФ, дивиденды Яндекса и Татнефти и другие новости недели - SberCIB</x:v>
       </x:c>
       <x:c r="AC35" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3497,22 +3501,22 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="41" t="str">
-        <x:v>DL-0bceebeca9933dc3</x:v>
+        <x:v>DL-6bc0569f7ac374fe</x:v>
       </x:c>
       <x:c r="B36" s="43" t="n">
-        <x:v>46132</x:v>
+        <x:v>46139</x:v>
       </x:c>
       <x:c r="C36" s="41" t="str">
-        <x:v>DCM</x:v>
+        <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D36" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E36" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="F36" s="41" t="str">
         <x:v>Ozon</x:v>
-      </x:c>
-      <x:c r="F36" s="41" t="str">
-        <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G36" s="41" t="str">
         <x:v>Financials</x:v>
@@ -3527,7 +3531,7 @@
       </x:c>
       <x:c r="L36" s="45"/>
       <x:c r="M36" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>Shares</x:v>
       </x:c>
       <x:c r="N36" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3547,7 +3551,7 @@
         <x:f>IFERROR(IF(AND($J36&gt;0,$P36&gt;0,$K36=$R36),$J36/$P36,""),"")</x:f>
       </x:c>
       <x:c r="U36" s="41" t="str">
-        <x:v>Bonds</x:v>
+        <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V36" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3562,13 +3566,13 @@
         <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z36" s="41" t="str">
-        <x:v>Альфа-Банк</x:v>
+        <x:v>Ведомости</x:v>
       </x:c>
       <x:c r="AA36" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMihgFBVV95cUxOR21Vd1RCOGpSRktSR2g3Mm11emdNTHVpLTlESXFfUVc5SFZFYkZYTWcwZ1kxc2ZUU1lPVWo3UmRjQXl4SFREaElpVTZvZktVMW43QXhNU2ZHal9hSHQ0bkttRV8xa1BVbHRHSENoSE5GblYwZElISUxNbG1fSG1uWUJ0QVgtZw?oc=5</x:v>
+        <x:v>https://www.vedomosti.ru/finance/news/2026/04/27/1193355-putin-isklyuchil</x:v>
       </x:c>
       <x:c r="AB36" s="41" t="str">
-        <x:v>Облигации Озона: заработай на маркетплейсе - Альфа-Банк</x:v>
+        <x:v>Путин исключил «Озон банк» из списка с запретом на сделки с акциями и долями - Ведомости</x:v>
       </x:c>
       <x:c r="AC36" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3576,10 +3580,10 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="41" t="str">
-        <x:v>DL-c10daba8af8e67d8</x:v>
+        <x:v>DL-cc671fa6b14f8f28</x:v>
       </x:c>
       <x:c r="B37" s="43" t="n">
-        <x:v>46128</x:v>
+        <x:v>46139</x:v>
       </x:c>
       <x:c r="C37" s="41" t="str">
         <x:v>M&amp;A</x:v>
@@ -3591,7 +3595,7 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F37" s="41" t="str">
-        <x:v>VK</x:v>
+        <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G37" s="41" t="str">
         <x:v>Financials</x:v>
@@ -3599,16 +3603,12 @@
       <x:c r="H37" s="41" t="str">
         <x:v>Not disclosed</x:v>
       </x:c>
-      <x:c r="I37" s="44" t="n">
-        <x:v>21200000000</x:v>
-      </x:c>
+      <x:c r="I37" s="44"/>
       <x:c r="J37" s="44"/>
       <x:c r="K37" s="41" t="str">
-        <x:v>RUB</x:v>
-      </x:c>
-      <x:c r="L37" s="45" t="n">
-        <x:v>0.25</x:v>
-      </x:c>
+        <x:v>NOT DISCLOSED</x:v>
+      </x:c>
+      <x:c r="L37" s="45"/>
       <x:c r="M37" s="41" t="str">
         <x:v>Shares</x:v>
       </x:c>
@@ -3636,22 +3636,22 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W37" s="41" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X37" s="41" t="str">
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y37" s="41" t="str">
-        <x:v>VKCO</x:v>
+        <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z37" s="41" t="str">
-        <x:v>RB.ru</x:v>
+        <x:v>БКС Экспресс</x:v>
       </x:c>
       <x:c r="AA37" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNQlJkLWo5eXZTSkZxSWU5NjF5TVJ0N1lYdXJqSzlFUGFMdk5jVEZMak1HeDE2SDZNcDduc3hENHkzaW8wWTVfWjN1QmpodGdYdDRLVXpua0pBUUs0MzVBX3lnOHlkVkJhVGdLNDlESDNRYmNmaDFaamJZVHdJRGhpX25lSkNmcmZ2dWZhZnhja2NwcXVnelJZVjg0Z1Flakd2VGl0MGRwUVdTTGtYYlNFcUYxSXdYaGY5?oc=5</x:v>
+        <x:v>https://bcs-express.ru/novosti-i-analitika/ozon-bank-iskliuchen-iz-perechnia-bankov-s-aktsiiami-kotorykh-zapreshcheny-sdelki</x:v>
       </x:c>
       <x:c r="AB37" s="41" t="str">
-        <x:v>VK продал 25% акций Точка Банка: сделку оценили в 21,2 млрд ₽ — вдвое выше изначальной стоимости бумаг - RB.ru</x:v>
+        <x:v>Ozon Банк исключен из перечня банков, с акциями которых запрещены сделки - БКС Экспресс</x:v>
       </x:c>
       <x:c r="AC37" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3659,10 +3659,10 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="41" t="str">
-        <x:v>DL-4d20ecb8f5c75dad</x:v>
+        <x:v>DL-2d1ef3023240f32a</x:v>
       </x:c>
       <x:c r="B38" s="43" t="n">
-        <x:v>46128</x:v>
+        <x:v>46139</x:v>
       </x:c>
       <x:c r="C38" s="41" t="str">
         <x:v>M&amp;A</x:v>
@@ -3674,24 +3674,22 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F38" s="41" t="str">
-        <x:v>VK</x:v>
+        <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G38" s="41" t="str">
         <x:v>Financials</x:v>
       </x:c>
       <x:c r="H38" s="41" t="str">
-        <x:v>Russia</x:v>
-      </x:c>
-      <x:c r="I38" s="44" t="n">
-        <x:v>21200000000</x:v>
-      </x:c>
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I38" s="44"/>
       <x:c r="J38" s="44"/>
       <x:c r="K38" s="41" t="str">
-        <x:v>RUB</x:v>
+        <x:v>NOT DISCLOSED</x:v>
       </x:c>
       <x:c r="L38" s="45"/>
       <x:c r="M38" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Shares</x:v>
       </x:c>
       <x:c r="N38" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3723,16 +3721,16 @@
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y38" s="41" t="str">
-        <x:v>VKCO</x:v>
+        <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z38" s="41" t="str">
-        <x:v>Ведомости</x:v>
+        <x:v>Главпортал</x:v>
       </x:c>
       <x:c r="AA38" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMifkFVX3lxTE1vSUlEOTl2cU5jckxzemNzN2oyNVZaX203N1VWRkpuZXNwYV9sdUNGMTZPTHhiNm5LWFBmdFM0QkFTRjFPczd4VEFlTEZpRzhiakF2ZGh5UU5kamRvbnFRTDE5dG8zOF9HRkk5MDUwVzBWbU9qWEN0MDhIdTJNUQ?oc=5</x:v>
+        <x:v>https://glavportal.com/news/putin-razreshil-sdelki-s-akciyami-ozon-banka</x:v>
       </x:c>
       <x:c r="AB38" s="41" t="str">
-        <x:v>VK продала долю в «Точка банке» по цене не менее 21,2 млрд рублей - Ведомости</x:v>
+        <x:v>Путин разрешил сделки с акциями «Озон банка» - Главпортал</x:v>
       </x:c>
       <x:c r="AC38" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3740,10 +3738,10 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="41" t="str">
-        <x:v>DL-dfc59ea0a0794532</x:v>
+        <x:v>DL-dd21f961f579e55a</x:v>
       </x:c>
       <x:c r="B39" s="43" t="n">
-        <x:v>46128</x:v>
+        <x:v>46139</x:v>
       </x:c>
       <x:c r="C39" s="41" t="str">
         <x:v>M&amp;A</x:v>
@@ -3755,7 +3753,7 @@
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="F39" s="41" t="str">
-        <x:v>VK</x:v>
+        <x:v>Ozon</x:v>
       </x:c>
       <x:c r="G39" s="41" t="str">
         <x:v>Financials</x:v>
@@ -3770,7 +3768,7 @@
       </x:c>
       <x:c r="L39" s="45"/>
       <x:c r="M39" s="41" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>Shares</x:v>
       </x:c>
       <x:c r="N39" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3793,7 +3791,7 @@
         <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V39" s="41" t="str">
-        <x:v>предпринимателей</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W39" s="41" t="n">
         <x:v>4</x:v>
@@ -3802,16 +3800,16 @@
         <x:v>unverified</x:v>
       </x:c>
       <x:c r="Y39" s="41" t="str">
-        <x:v>VKCO</x:v>
+        <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z39" s="41" t="str">
-        <x:v>CNews.ru</x:v>
+        <x:v>Реальное время</x:v>
       </x:c>
       <x:c r="AA39" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMigAFBVV95cUxOeU1NOHJNay1uUm9TdlpGcWh4YkNXN3J0clFCT2JrM0t5T3hwTmtTRlJXUWpyeVBYbnltZlB0dnpqLWxhTUxQNW9wQU1LeG5sTjVzT1NNQlFlY0Jpb1REMGhyWG1wSUM0STZXbFFaNndzQ1A1MlVvMFN3RmlmOW4tXw?oc=5</x:v>
+        <x:v>https://realnoevremya.ru/news/394463-s-ozon-banka-snyali-ogranicheniya-na-sdelki-s-akciyami-rasporyazhenie-putina</x:v>
       </x:c>
       <x:c r="AB39" s="41" t="str">
-        <x:v>VK продал свою долю в виртуальном банке для предпринимателей - CNews.ru</x:v>
+        <x:v>С «Озон банка» сняли ограничения на сделки с акциями — распоряжение Путина - Реальное время</x:v>
       </x:c>
       <x:c r="AC39" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3819,39 +3817,37 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="41" t="str">
-        <x:v>DL-1363a495ec14164a</x:v>
+        <x:v>DL-09b72d880f67361b</x:v>
       </x:c>
       <x:c r="B40" s="43" t="n">
-        <x:v>46115</x:v>
+        <x:v>46139</x:v>
       </x:c>
       <x:c r="C40" s="41" t="str">
-        <x:v>DCM</x:v>
+        <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D40" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E40" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="F40" s="41" t="str">
         <x:v>Ozon</x:v>
       </x:c>
-      <x:c r="F40" s="41" t="str">
-        <x:v>Not applicable</x:v>
-      </x:c>
       <x:c r="G40" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Financials</x:v>
       </x:c>
       <x:c r="H40" s="41" t="str">
         <x:v>Russia</x:v>
       </x:c>
-      <x:c r="I40" s="44" t="n">
-        <x:v>15000000000</x:v>
-      </x:c>
+      <x:c r="I40" s="44"/>
       <x:c r="J40" s="44"/>
       <x:c r="K40" s="41" t="str">
-        <x:v>RUB</x:v>
+        <x:v>NOT DISCLOSED</x:v>
       </x:c>
       <x:c r="L40" s="45"/>
       <x:c r="M40" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>Shares</x:v>
       </x:c>
       <x:c r="N40" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3871,7 +3867,7 @@
         <x:f>IFERROR(IF(AND($J40&gt;0,$P40&gt;0,$K40=$R40),$J40/$P40,""),"")</x:f>
       </x:c>
       <x:c r="U40" s="41" t="str">
-        <x:v>Bonds</x:v>
+        <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V40" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3886,13 +3882,13 @@
         <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z40" s="41" t="str">
-        <x:v>https://expert.ru</x:v>
+        <x:v>InvestFuture</x:v>
       </x:c>
       <x:c r="AA40" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiigFBVV95cUxNVmVRdkQ4RElHdURKbmVDQU9NbVRmZTd0Z3NiM3JzMjFhZzNzQzVPMnhzNHFER2VsYVAyWEpwVlg4c24zZUozY1ZNUFQxNDMxakR1Q1J0RFhhbkRxbUZYTmgtc3N3UzhsckljT1lpZTFvaXJKeGlTblNyNlNWb2JhOWFSVXZJWjZ0Rmc?oc=5</x:v>
+        <x:v>https://investfuture.ru/articles/putin-snyal-zapret-na-sdelki-s-aktsiyami-ozon-banka-v-rossii-1178931397</x:v>
       </x:c>
       <x:c r="AB40" s="41" t="str">
-        <x:v>Ozon анонсировал размещение облигаций на 15 млрд рублей - https://expert.ru</x:v>
+        <x:v>Путин снял запрет на сделки с акциями Озон банка в России | IF | 27.04.2026 - InvestFuture</x:v>
       </x:c>
       <x:c r="AC40" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3900,16 +3896,16 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="41" t="str">
-        <x:v>DL-12855c6275c496fe</x:v>
+        <x:v>DL-0bceebeca9933dc3</x:v>
       </x:c>
       <x:c r="B41" s="43" t="n">
-        <x:v>46115</x:v>
+        <x:v>46132</x:v>
       </x:c>
       <x:c r="C41" s="41" t="str">
         <x:v>DCM</x:v>
       </x:c>
       <x:c r="D41" s="41" t="str">
-        <x:v>Announced</x:v>
+        <x:v>Reported</x:v>
       </x:c>
       <x:c r="E41" s="41" t="str">
         <x:v>Ozon</x:v>
@@ -3918,7 +3914,7 @@
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="G41" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Financials</x:v>
       </x:c>
       <x:c r="H41" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -3965,13 +3961,13 @@
         <x:v>OZON</x:v>
       </x:c>
       <x:c r="Z41" s="41" t="str">
-        <x:v>БКС Экспресс</x:v>
+        <x:v>Альфа-Банк</x:v>
       </x:c>
       <x:c r="AA41" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMipgFBVV95cUxNTmtrN3N0YVN0c0NuVnBscUJvbzdVbWZ5OXczRTkySkx1T1hKdWJvZlFWNEFqbkxhRmpXVEVQZUdIcjdOZkNFRnJhX1huRGRmelhla1RRTURfejMzd2FIMU9ZcmQ4REtOWWEyZ3JhLUgwSmI2UDhJM2s4TkNRekY0T3ZtcEJNbUYzNTQzOXRITGxsN1A0N1duQ3FKeE5fTXIxMUVJTlh3?oc=5</x:v>
+        <x:v>https://alfabank.ru/alfa-investor/t/obligatsii-ozona-zarabotay-na-marketpleyse/</x:v>
       </x:c>
       <x:c r="AB41" s="41" t="str">
-        <x:v>Озон планирует дебютное размещение биржевых облигаций - БКС Экспресс</x:v>
+        <x:v>Облигации Озона: заработай на маркетплейсе - Альфа-Банк</x:v>
       </x:c>
       <x:c r="AC41" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -3979,39 +3975,41 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="41" t="str">
-        <x:v>DL-d39c99c4c2dfa45c</x:v>
+        <x:v>DL-c10daba8af8e67d8</x:v>
       </x:c>
       <x:c r="B42" s="43" t="n">
-        <x:v>46111</x:v>
+        <x:v>46128</x:v>
       </x:c>
       <x:c r="C42" s="41" t="str">
-        <x:v>DCM</x:v>
+        <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D42" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E42" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="F42" s="41" t="str">
         <x:v>VK</x:v>
       </x:c>
-      <x:c r="F42" s="41" t="str">
-        <x:v>Not applicable</x:v>
-      </x:c>
       <x:c r="G42" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Financials</x:v>
       </x:c>
       <x:c r="H42" s="41" t="str">
-        <x:v>Russia</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="I42" s="44" t="n">
-        <x:v>10000000000</x:v>
+        <x:v>21200000000</x:v>
       </x:c>
       <x:c r="J42" s="44"/>
       <x:c r="K42" s="41" t="str">
         <x:v>RUB</x:v>
       </x:c>
-      <x:c r="L42" s="45"/>
+      <x:c r="L42" s="45" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
       <x:c r="M42" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>Shares</x:v>
       </x:c>
       <x:c r="N42" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -4031,13 +4029,13 @@
         <x:f>IFERROR(IF(AND($J42&gt;0,$P42&gt;0,$K42=$R42),$J42/$P42,""),"")</x:f>
       </x:c>
       <x:c r="U42" s="41" t="str">
-        <x:v>Bonds</x:v>
+        <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V42" s="41" t="str">
         <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="W42" s="41" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="X42" s="41" t="str">
         <x:v>unverified</x:v>
@@ -4046,13 +4044,13 @@
         <x:v>VKCO</x:v>
       </x:c>
       <x:c r="Z42" s="41" t="str">
-        <x:v>vk.company</x:v>
+        <x:v>RB.ru</x:v>
       </x:c>
       <x:c r="AA42" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE1WcXUxeUFkWFdQQUk3U0o0RDBfeTdxa3IxV0dWLXRZZXRjWWo1M0NBOUJfeVUwNHRuMUxaOVBKVXdjSWstd1paRHFfX2lpT1VpV0E?oc=5</x:v>
+        <x:v>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNQlJkLWo5eXZTSkZxSWU5NjF5TVJ0N1lYdXJqSzlFUGFMdk5jVEZMak1HeDE2SDZNcDduc3hENHkzaW8wWTVfWjN1QmpodGdYdDRLVXpua0pBUUs0MzVBX3lnOHlkVkJhVGdLNDlESDNRYmNmaDFaamJZVHdJRGhpX25lSkNmcmZ2dWZhZnhja2NwcXVnelJZVjg0Z1Flakd2VGl0MGRwUVdTTGtYYlNFcUYxSXdYaGY5?oc=5</x:v>
       </x:c>
       <x:c r="AB42" s="41" t="str">
-        <x:v>VK объявляет о планах по размещению биржевых облигаций объемом 10 млрд рублей - vk.company</x:v>
+        <x:v>VK продал 25% акций Точка Банка: сделку оценили в 21,2 млрд ₽ — вдвое выше изначальной стоимости бумаг - RB.ru</x:v>
       </x:c>
       <x:c r="AC42" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
@@ -4060,37 +4058,39 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="41" t="str">
-        <x:v>DL-b9babb23f2c4462c</x:v>
+        <x:v>DL-4d20ecb8f5c75dad</x:v>
       </x:c>
       <x:c r="B43" s="43" t="n">
-        <x:v>46111</x:v>
+        <x:v>46128</x:v>
       </x:c>
       <x:c r="C43" s="41" t="str">
-        <x:v>DCM</x:v>
+        <x:v>M&amp;A</x:v>
       </x:c>
       <x:c r="D43" s="41" t="str">
         <x:v>Reported</x:v>
       </x:c>
       <x:c r="E43" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="F43" s="41" t="str">
         <x:v>VK</x:v>
       </x:c>
-      <x:c r="F43" s="41" t="str">
-        <x:v>Not applicable</x:v>
-      </x:c>
       <x:c r="G43" s="41" t="str">
-        <x:v>Not classified</x:v>
+        <x:v>Financials</x:v>
       </x:c>
       <x:c r="H43" s="41" t="str">
-        <x:v>Not disclosed</x:v>
-      </x:c>
-      <x:c r="I43" s="44"/>
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I43" s="44" t="n">
+        <x:v>21200000000</x:v>
+      </x:c>
       <x:c r="J43" s="44"/>
       <x:c r="K43" s="41" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
       <x:c r="L43" s="45"/>
       <x:c r="M43" s="41" t="str">
-        <x:v>Not applicable</x:v>
+        <x:v>Not disclosed</x:v>
       </x:c>
       <x:c r="N43" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -4110,7 +4110,7 @@
         <x:f>IFERROR(IF(AND($J43&gt;0,$P43&gt;0,$K43=$R43),$J43/$P43,""),"")</x:f>
       </x:c>
       <x:c r="U43" s="41" t="str">
-        <x:v>Bonds</x:v>
+        <x:v>Acquisition / disposal</x:v>
       </x:c>
       <x:c r="V43" s="41" t="str">
         <x:v>Not disclosed</x:v>
@@ -4125,15 +4125,1050 @@
         <x:v>VKCO</x:v>
       </x:c>
       <x:c r="Z43" s="41" t="str">
+        <x:v>Ведомости</x:v>
+      </x:c>
+      <x:c r="AA43" s="41" t="str">
+        <x:v>https://news.google.com/rss/articles/CBMifkFVX3lxTE1vSUlEOTl2cU5jckxzemNzN2oyNVZaX203N1VWRkpuZXNwYV9sdUNGMTZPTHhiNm5LWFBmdFM0QkFTRjFPczd4VEFlTEZpRzhiakF2ZGh5UU5kamRvbnFRTDE5dG8zOF9HRkk5MDUwVzBWbU9qWEN0MDhIdTJNUQ?oc=5</x:v>
+      </x:c>
+      <x:c r="AB43" s="41" t="str">
+        <x:v>VK продала долю в «Точка банке» по цене не менее 21,2 млрд рублей - Ведомости</x:v>
+      </x:c>
+      <x:c r="AC43" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="41" t="str">
+        <x:v>DL-dfc59ea0a0794532</x:v>
+      </x:c>
+      <x:c r="B44" s="43" t="n">
+        <x:v>46128</x:v>
+      </x:c>
+      <x:c r="C44" s="41" t="str">
+        <x:v>M&amp;A</x:v>
+      </x:c>
+      <x:c r="D44" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E44" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="F44" s="41" t="str">
+        <x:v>VK</x:v>
+      </x:c>
+      <x:c r="G44" s="41" t="str">
+        <x:v>Financials</x:v>
+      </x:c>
+      <x:c r="H44" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I44" s="44"/>
+      <x:c r="J44" s="44"/>
+      <x:c r="K44" s="41" t="str">
+        <x:v>NOT DISCLOSED</x:v>
+      </x:c>
+      <x:c r="L44" s="45"/>
+      <x:c r="M44" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="N44" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O44" s="44"/>
+      <x:c r="P44" s="44"/>
+      <x:c r="Q44" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R44" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S44" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J44&gt;0,$O44&gt;0,$K44=$R44),$J44/$O44,""),"")</x:f>
+      </x:c>
+      <x:c r="T44" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J44&gt;0,$P44&gt;0,$K44=$R44),$J44/$P44,""),"")</x:f>
+      </x:c>
+      <x:c r="U44" s="41" t="str">
+        <x:v>Acquisition / disposal</x:v>
+      </x:c>
+      <x:c r="V44" s="41" t="str">
+        <x:v>предпринимателей</x:v>
+      </x:c>
+      <x:c r="W44" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="X44" s="41" t="str">
+        <x:v>unverified</x:v>
+      </x:c>
+      <x:c r="Y44" s="41" t="str">
+        <x:v>VKCO</x:v>
+      </x:c>
+      <x:c r="Z44" s="41" t="str">
+        <x:v>CNews.ru</x:v>
+      </x:c>
+      <x:c r="AA44" s="41" t="str">
+        <x:v>https://news.google.com/rss/articles/CBMigAFBVV95cUxOeU1NOHJNay1uUm9TdlpGcWh4YkNXN3J0clFCT2JrM0t5T3hwTmtTRlJXUWpyeVBYbnltZlB0dnpqLWxhTUxQNW9wQU1LeG5sTjVzT1NNQlFlY0Jpb1REMGhyWG1wSUM0STZXbFFaNndzQ1A1MlVvMFN3RmlmOW4tXw?oc=5</x:v>
+      </x:c>
+      <x:c r="AB44" s="41" t="str">
+        <x:v>VK продал свою долю в виртуальном банке для предпринимателей - CNews.ru</x:v>
+      </x:c>
+      <x:c r="AC44" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="41" t="str">
+        <x:v>DL-4774de17c61c14e4</x:v>
+      </x:c>
+      <x:c r="B45" s="43" t="n">
+        <x:v>46122</x:v>
+      </x:c>
+      <x:c r="C45" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D45" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E45" s="41" t="str">
+        <x:v>VK</x:v>
+      </x:c>
+      <x:c r="F45" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G45" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H45" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I45" s="44"/>
+      <x:c r="J45" s="44"/>
+      <x:c r="K45" s="41" t="str">
+        <x:v>NOT DISCLOSED</x:v>
+      </x:c>
+      <x:c r="L45" s="45"/>
+      <x:c r="M45" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N45" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O45" s="44"/>
+      <x:c r="P45" s="44"/>
+      <x:c r="Q45" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R45" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S45" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J45&gt;0,$O45&gt;0,$K45=$R45),$J45/$O45,""),"")</x:f>
+      </x:c>
+      <x:c r="T45" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J45&gt;0,$P45&gt;0,$K45=$R45),$J45/$P45,""),"")</x:f>
+      </x:c>
+      <x:c r="U45" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V45" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W45" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="X45" s="41" t="str">
+        <x:v>unverified</x:v>
+      </x:c>
+      <x:c r="Y45" s="41" t="str">
+        <x:v>VKCO</x:v>
+      </x:c>
+      <x:c r="Z45" s="41" t="str">
         <x:v>Финам</x:v>
       </x:c>
-      <x:c r="AA43" s="41" t="str">
-        <x:v>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPR3ZFSWgwcm9TTW9rSTlBM0VaYncwM3dBZ0N0OUhwWFBnYVZLc3EtZkNrOE5RLUFjczJ5b25yNURHX0RvYkNPbUFfTlhiSkU3U185NFM0b3R3ZVJVbVEweXI4Q1hRVDBwN3dlcHpocDFYTmRYalh4d1Q1RVU3M1JHZ18ydXdQc2s0OUJGQTJwOFRydlNZOTNJbkItdEtZQVRyb3BMWU5fY082ZHZzbDdNbmNRZWJHRUVhd0FIUkhtX28?oc=5</x:v>
-      </x:c>
-      <x:c r="AB43" s="41" t="str">
+      <x:c r="AA45" s="41" t="str">
+        <x:v>https://www.finam.ru/publications/item/dvoynoe-razmeshchenie-obligatsiy-vk-chego-zhdat-chastnym-investoram-20260410-1829/</x:v>
+      </x:c>
+      <x:c r="AB45" s="41" t="str">
+        <x:v>Двойное размещение облигаций VK. Чего ждать частным инвесторам? 10.04.2026 - Финам</x:v>
+      </x:c>
+      <x:c r="AC45" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="41" t="str">
+        <x:v>DL-87f81143148d7276</x:v>
+      </x:c>
+      <x:c r="B46" s="43" t="n">
+        <x:v>46122</x:v>
+      </x:c>
+      <x:c r="C46" s="41" t="str">
+        <x:v>ECM</x:v>
+      </x:c>
+      <x:c r="D46" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E46" s="41" t="str">
+        <x:v>Ozon</x:v>
+      </x:c>
+      <x:c r="F46" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G46" s="41" t="str">
+        <x:v>Financials</x:v>
+      </x:c>
+      <x:c r="H46" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I46" s="44"/>
+      <x:c r="J46" s="44"/>
+      <x:c r="K46" s="41" t="str">
+        <x:v>NOT DISCLOSED</x:v>
+      </x:c>
+      <x:c r="L46" s="45"/>
+      <x:c r="M46" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N46" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O46" s="44"/>
+      <x:c r="P46" s="44"/>
+      <x:c r="Q46" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R46" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S46" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J46&gt;0,$O46&gt;0,$K46=$R46),$J46/$O46,""),"")</x:f>
+      </x:c>
+      <x:c r="T46" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J46&gt;0,$P46&gt;0,$K46=$R46),$J46/$P46,""),"")</x:f>
+      </x:c>
+      <x:c r="U46" s="41" t="str">
+        <x:v>Equity issuance</x:v>
+      </x:c>
+      <x:c r="V46" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W46" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="X46" s="41" t="str">
+        <x:v>unverified</x:v>
+      </x:c>
+      <x:c r="Y46" s="41" t="str">
+        <x:v>OZON</x:v>
+      </x:c>
+      <x:c r="Z46" s="41" t="str">
+        <x:v>Альфа-Банк</x:v>
+      </x:c>
+      <x:c r="AA46" s="41" t="str">
+        <x:v>https://news.google.com/rss/articles/CBMihgFBVV95cUxNbVZjUURpZDgxcTE2VG9jRktkMVZHRmpqSG9jclBJZU45SVNzS3VLTUFyYkhnUWdpQl9pb1Jvd1p5Ni12Z1pFQWlKeDQtUDUxY0xCSVA0dno3ZjJzWnZkS3RLVWh3UjNGWVJXd29rbjFBUjdVUnZwa1RGdk9hQTIxMHBCRzFPdw?oc=5</x:v>
+      </x:c>
+      <x:c r="AB46" s="41" t="str">
+        <x:v>Мы держим Ozon в портфеле роста, но не в дивидендном Хотя - Альфа-Банк</x:v>
+      </x:c>
+      <x:c r="AC46" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="41" t="str">
+        <x:v>DL-1363a495ec14164a</x:v>
+      </x:c>
+      <x:c r="B47" s="43" t="n">
+        <x:v>46115</x:v>
+      </x:c>
+      <x:c r="C47" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D47" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E47" s="41" t="str">
+        <x:v>Ozon</x:v>
+      </x:c>
+      <x:c r="F47" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G47" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H47" s="41" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I47" s="44" t="n">
+        <x:v>15000000000</x:v>
+      </x:c>
+      <x:c r="J47" s="44"/>
+      <x:c r="K47" s="41" t="str">
+        <x:v>RUB</x:v>
+      </x:c>
+      <x:c r="L47" s="45"/>
+      <x:c r="M47" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N47" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O47" s="44"/>
+      <x:c r="P47" s="44"/>
+      <x:c r="Q47" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R47" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S47" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J47&gt;0,$O47&gt;0,$K47=$R47),$J47/$O47,""),"")</x:f>
+      </x:c>
+      <x:c r="T47" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J47&gt;0,$P47&gt;0,$K47=$R47),$J47/$P47,""),"")</x:f>
+      </x:c>
+      <x:c r="U47" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V47" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W47" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="X47" s="41" t="str">
+        <x:v>unverified</x:v>
+      </x:c>
+      <x:c r="Y47" s="41" t="str">
+        <x:v>OZON</x:v>
+      </x:c>
+      <x:c r="Z47" s="41" t="str">
+        <x:v>https://expert.ru</x:v>
+      </x:c>
+      <x:c r="AA47" s="41" t="str">
+        <x:v>https://news.google.com/rss/articles/CBMiigFBVV95cUxNVmVRdkQ4RElHdURKbmVDQU9NbVRmZTd0Z3NiM3JzMjFhZzNzQzVPMnhzNHFER2VsYVAyWEpwVlg4c24zZUozY1ZNUFQxNDMxakR1Q1J0RFhhbkRxbUZYTmgtc3N3UzhsckljT1lpZTFvaXJKeGlTblNyNlNWb2JhOWFSVXZJWjZ0Rmc?oc=5</x:v>
+      </x:c>
+      <x:c r="AB47" s="41" t="str">
+        <x:v>Ozon анонсировал размещение облигаций на 15 млрд рублей - https://expert.ru</x:v>
+      </x:c>
+      <x:c r="AC47" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="41" t="str">
+        <x:v>DL-12855c6275c496fe</x:v>
+      </x:c>
+      <x:c r="B48" s="43" t="n">
+        <x:v>46115</x:v>
+      </x:c>
+      <x:c r="C48" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D48" s="41" t="str">
+        <x:v>Announced</x:v>
+      </x:c>
+      <x:c r="E48" s="41" t="str">
+        <x:v>Ozon</x:v>
+      </x:c>
+      <x:c r="F48" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G48" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H48" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I48" s="44"/>
+      <x:c r="J48" s="44"/>
+      <x:c r="K48" s="41" t="str">
+        <x:v>NOT DISCLOSED</x:v>
+      </x:c>
+      <x:c r="L48" s="45"/>
+      <x:c r="M48" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N48" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O48" s="44"/>
+      <x:c r="P48" s="44"/>
+      <x:c r="Q48" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R48" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S48" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J48&gt;0,$O48&gt;0,$K48=$R48),$J48/$O48,""),"")</x:f>
+      </x:c>
+      <x:c r="T48" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J48&gt;0,$P48&gt;0,$K48=$R48),$J48/$P48,""),"")</x:f>
+      </x:c>
+      <x:c r="U48" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V48" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W48" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="X48" s="41" t="str">
+        <x:v>unverified</x:v>
+      </x:c>
+      <x:c r="Y48" s="41" t="str">
+        <x:v>OZON</x:v>
+      </x:c>
+      <x:c r="Z48" s="41" t="str">
+        <x:v>БКС Экспресс</x:v>
+      </x:c>
+      <x:c r="AA48" s="41" t="str">
+        <x:v>https://news.google.com/rss/articles/CBMipgFBVV95cUxNTmtrN3N0YVN0c0NuVnBscUJvbzdVbWZ5OXczRTkySkx1T1hKdWJvZlFWNEFqbkxhRmpXVEVQZUdIcjdOZkNFRnJhX1huRGRmelhla1RRTURfejMzd2FIMU9ZcmQ4REtOWWEyZ3JhLUgwSmI2UDhJM2s4TkNRekY0T3ZtcEJNbUYzNTQzOXRITGxsN1A0N1duQ3FKeE5fTXIxMUVJTlh3?oc=5</x:v>
+      </x:c>
+      <x:c r="AB48" s="41" t="str">
+        <x:v>Озон планирует дебютное размещение биржевых облигаций - БКС Экспресс</x:v>
+      </x:c>
+      <x:c r="AC48" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="41" t="str">
+        <x:v>DL-d39c99c4c2dfa45c</x:v>
+      </x:c>
+      <x:c r="B49" s="43" t="n">
+        <x:v>46111</x:v>
+      </x:c>
+      <x:c r="C49" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D49" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E49" s="41" t="str">
+        <x:v>VK</x:v>
+      </x:c>
+      <x:c r="F49" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G49" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H49" s="41" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I49" s="44" t="n">
+        <x:v>10000000000</x:v>
+      </x:c>
+      <x:c r="J49" s="44"/>
+      <x:c r="K49" s="41" t="str">
+        <x:v>RUB</x:v>
+      </x:c>
+      <x:c r="L49" s="45"/>
+      <x:c r="M49" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N49" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O49" s="44"/>
+      <x:c r="P49" s="44"/>
+      <x:c r="Q49" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R49" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S49" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J49&gt;0,$O49&gt;0,$K49=$R49),$J49/$O49,""),"")</x:f>
+      </x:c>
+      <x:c r="T49" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J49&gt;0,$P49&gt;0,$K49=$R49),$J49/$P49,""),"")</x:f>
+      </x:c>
+      <x:c r="U49" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V49" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W49" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="X49" s="41" t="str">
+        <x:v>unverified</x:v>
+      </x:c>
+      <x:c r="Y49" s="41" t="str">
+        <x:v>VKCO</x:v>
+      </x:c>
+      <x:c r="Z49" s="41" t="str">
+        <x:v>vk.company</x:v>
+      </x:c>
+      <x:c r="AA49" s="41" t="str">
+        <x:v>https://news.google.com/rss/articles/CBMiUkFVX3lxTE1WcXUxeUFkWFdQQUk3U0o0RDBfeTdxa3IxV0dWLXRZZXRjWWo1M0NBOUJfeVUwNHRuMUxaOVBKVXdjSWstd1paRHFfX2lpT1VpV0E?oc=5</x:v>
+      </x:c>
+      <x:c r="AB49" s="41" t="str">
+        <x:v>VK объявляет о планах по размещению биржевых облигаций объемом 10 млрд рублей - vk.company</x:v>
+      </x:c>
+      <x:c r="AC49" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="41" t="str">
+        <x:v>DL-b9babb23f2c4462c</x:v>
+      </x:c>
+      <x:c r="B50" s="43" t="n">
+        <x:v>46111</x:v>
+      </x:c>
+      <x:c r="C50" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D50" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E50" s="41" t="str">
+        <x:v>VK</x:v>
+      </x:c>
+      <x:c r="F50" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G50" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H50" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I50" s="44"/>
+      <x:c r="J50" s="44"/>
+      <x:c r="K50" s="41" t="str">
+        <x:v>NOT DISCLOSED</x:v>
+      </x:c>
+      <x:c r="L50" s="45"/>
+      <x:c r="M50" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N50" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O50" s="44"/>
+      <x:c r="P50" s="44"/>
+      <x:c r="Q50" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R50" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S50" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J50&gt;0,$O50&gt;0,$K50=$R50),$J50/$O50,""),"")</x:f>
+      </x:c>
+      <x:c r="T50" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J50&gt;0,$P50&gt;0,$K50=$R50),$J50/$P50,""),"")</x:f>
+      </x:c>
+      <x:c r="U50" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V50" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W50" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="X50" s="41" t="str">
+        <x:v>unverified</x:v>
+      </x:c>
+      <x:c r="Y50" s="41" t="str">
+        <x:v>VKCO</x:v>
+      </x:c>
+      <x:c r="Z50" s="41" t="str">
+        <x:v>Финам</x:v>
+      </x:c>
+      <x:c r="AA50" s="41" t="str">
+        <x:v>https://www.finam.ru/publications/item/vk-razmeshchaet-obligatsii-kak-eto-otrazitsya-na-investorakh-v-aktsii-20260330-1740/</x:v>
+      </x:c>
+      <x:c r="AB50" s="41" t="str">
         <x:v>VK размещает облигации: как это отразится на инвесторах в акции 30.03.2026 - Финам</x:v>
       </x:c>
-      <x:c r="AC43" s="41" t="str">
+      <x:c r="AC50" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="41" t="str">
+        <x:v>DL-238a83afad61e805</x:v>
+      </x:c>
+      <x:c r="B51" s="43" t="n">
+        <x:v>46080</x:v>
+      </x:c>
+      <x:c r="C51" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D51" s="41" t="str">
+        <x:v>Issued</x:v>
+      </x:c>
+      <x:c r="E51" s="41" t="str">
+        <x:v>SELECTEL</x:v>
+      </x:c>
+      <x:c r="F51" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G51" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H51" s="41" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I51" s="44" t="n">
+        <x:v>7000000000</x:v>
+      </x:c>
+      <x:c r="J51" s="44"/>
+      <x:c r="K51" s="41" t="str">
+        <x:v>RUB</x:v>
+      </x:c>
+      <x:c r="L51" s="45" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="M51" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N51" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O51" s="44"/>
+      <x:c r="P51" s="44"/>
+      <x:c r="Q51" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R51" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S51" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J51&gt;0,$O51&gt;0,$K51=$R51),$J51/$O51,""),"")</x:f>
+      </x:c>
+      <x:c r="T51" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J51&gt;0,$P51&gt;0,$K51=$R51),$J51/$P51,""),"")</x:f>
+      </x:c>
+      <x:c r="U51" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V51" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W51" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="X51" s="41" t="str">
+        <x:v>confirmed</x:v>
+      </x:c>
+      <x:c r="Y51" s="41" t="str"/>
+      <x:c r="Z51" s="41" t="str">
+        <x:v>Selectel Newsroom</x:v>
+      </x:c>
+      <x:c r="AA51" s="41" t="str">
+        <x:v>https://selectel.ru/about/newsroom/news/selectel-razmestil-novyj-vypusk-obligaczij-i-privlek-7-milliardov-rublej-na-razvitie-biznesa/</x:v>
+      </x:c>
+      <x:c r="AB51" s="41" t="str">
+        <x:v>Selectel разместил новый выпуск облигаций и привлек 7 миллиардов рублей на развитие бизнеса Selectel сообщил об успешном закрытии книги заявок в рамках размещения выпуска облигаций серии 001P-07R по ставке купона 15,00% годовых сроком на три года. В ходе формирования книги заявок общий спрос инвесторов превысил первоначальный ориентир по объему выпуска, что позволило увеличить объем выпуска с 5 до 7 млрд рублей и снизить итоговую ставку купона до 15,00% годовых.</x:v>
+      </x:c>
+      <x:c r="AC51" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="41" t="str">
+        <x:v>DL-251bf0d0b7b600c1</x:v>
+      </x:c>
+      <x:c r="B52" s="43" t="n">
+        <x:v>45642</x:v>
+      </x:c>
+      <x:c r="C52" s="41" t="str">
+        <x:v>M&amp;A</x:v>
+      </x:c>
+      <x:c r="D52" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E52" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="F52" s="41" t="str">
+        <x:v>SELECTEL</x:v>
+      </x:c>
+      <x:c r="G52" s="41" t="str">
+        <x:v>Technology</x:v>
+      </x:c>
+      <x:c r="H52" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="I52" s="44"/>
+      <x:c r="J52" s="44"/>
+      <x:c r="K52" s="41" t="str">
+        <x:v>NOT DISCLOSED</x:v>
+      </x:c>
+      <x:c r="L52" s="45" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M52" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="N52" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O52" s="44"/>
+      <x:c r="P52" s="44"/>
+      <x:c r="Q52" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R52" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S52" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J52&gt;0,$O52&gt;0,$K52=$R52),$J52/$O52,""),"")</x:f>
+      </x:c>
+      <x:c r="T52" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J52&gt;0,$P52&gt;0,$K52=$R52),$J52/$P52,""),"")</x:f>
+      </x:c>
+      <x:c r="U52" s="41" t="str">
+        <x:v>Acquisition / disposal</x:v>
+      </x:c>
+      <x:c r="V52" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W52" s="41" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="X52" s="41" t="str">
+        <x:v>confirmed</x:v>
+      </x:c>
+      <x:c r="Y52" s="41" t="str"/>
+      <x:c r="Z52" s="41" t="str">
+        <x:v>Selectel Newsroom</x:v>
+      </x:c>
+      <x:c r="AA52" s="41" t="str">
+        <x:v>https://selectel.ru/about/newsroom/news/selectel-soobshchaet-o-priobretenii-oblachnogo-provajdera-servers-ru/</x:v>
+      </x:c>
+      <x:c r="AB52" s="41" t="str">
+        <x:v>Selectel сообщает о приобретении облачного провайдера Servers.ru Selectel сообщает о приобретении 100% компании ООО «Единая сеть», работающей под брендами Servers.ru, Exepto.ru и Fozzy.ru. Сделка позволит ускорить рост бизнеса и усилить лидерские позиции Selectel на рынке облачных инфраструктурных сервисов.</x:v>
+      </x:c>
+      <x:c r="AC52" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="41" t="str">
+        <x:v>DL-aa5a93661389a659</x:v>
+      </x:c>
+      <x:c r="B53" s="43" t="n">
+        <x:v>45611</x:v>
+      </x:c>
+      <x:c r="C53" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D53" s="41" t="str">
+        <x:v>Announced</x:v>
+      </x:c>
+      <x:c r="E53" s="41" t="str">
+        <x:v>SELECTEL</x:v>
+      </x:c>
+      <x:c r="F53" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G53" s="41" t="str">
+        <x:v>Financials</x:v>
+      </x:c>
+      <x:c r="H53" s="41" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I53" s="44" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="J53" s="44"/>
+      <x:c r="K53" s="41" t="str">
+        <x:v>RUB</x:v>
+      </x:c>
+      <x:c r="L53" s="45"/>
+      <x:c r="M53" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N53" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O53" s="44"/>
+      <x:c r="P53" s="44"/>
+      <x:c r="Q53" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R53" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S53" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J53&gt;0,$O53&gt;0,$K53=$R53),$J53/$O53,""),"")</x:f>
+      </x:c>
+      <x:c r="T53" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J53&gt;0,$P53&gt;0,$K53=$R53),$J53/$P53,""),"")</x:f>
+      </x:c>
+      <x:c r="U53" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V53" s="41" t="str">
+        <x:v>целей финансирования инвестиционной программы</x:v>
+      </x:c>
+      <x:c r="W53" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="X53" s="41" t="str">
+        <x:v>confirmed</x:v>
+      </x:c>
+      <x:c r="Y53" s="41" t="str"/>
+      <x:c r="Z53" s="41" t="str">
+        <x:v>Selectel Newsroom</x:v>
+      </x:c>
+      <x:c r="AA53" s="41" t="str">
+        <x:v>https://selectel.ru/about/newsroom/news/selectel-planiruet-razmeshhenie-obligaczij-obemom-3-milliarda-rublej-2/</x:v>
+      </x:c>
+      <x:c r="AB53" s="41" t="str">
+        <x:v>Selectel планирует размещение облигаций объемом 3 миллиарда рублей Компания Selectel планирует разместить новый выпуск облигаций объемом 3 млрд рублей для целей финансирования инвестиционной программы. Тип купона — переменный и определяется исходя из ключевой ставки Банка России плюс премия не выше 400 базисных пунктов. Срок обращения — 2,5 года с ежемесячной выплатой купона. Сбор заявок планируется провести в конце ноября.</x:v>
+      </x:c>
+      <x:c r="AC53" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="41" t="str">
+        <x:v>DL-c898acc93d60813b</x:v>
+      </x:c>
+      <x:c r="B54" s="43" t="n">
+        <x:v>45391</x:v>
+      </x:c>
+      <x:c r="C54" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D54" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E54" s="41" t="str">
+        <x:v>SELECTEL</x:v>
+      </x:c>
+      <x:c r="F54" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G54" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H54" s="41" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I54" s="44" t="n">
+        <x:v>4000000000</x:v>
+      </x:c>
+      <x:c r="J54" s="44"/>
+      <x:c r="K54" s="41" t="str">
+        <x:v>RUB</x:v>
+      </x:c>
+      <x:c r="L54" s="45" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="M54" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N54" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O54" s="44"/>
+      <x:c r="P54" s="44"/>
+      <x:c r="Q54" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R54" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S54" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J54&gt;0,$O54&gt;0,$K54=$R54),$J54/$O54,""),"")</x:f>
+      </x:c>
+      <x:c r="T54" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J54&gt;0,$P54&gt;0,$K54=$R54),$J54/$P54,""),"")</x:f>
+      </x:c>
+      <x:c r="U54" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V54" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W54" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="X54" s="41" t="str">
+        <x:v>confirmed</x:v>
+      </x:c>
+      <x:c r="Y54" s="41" t="str"/>
+      <x:c r="Z54" s="41" t="str">
+        <x:v>Selectel Newsroom</x:v>
+      </x:c>
+      <x:c r="AA54" s="41" t="str">
+        <x:v>https://selectel.ru/about/newsroom/news/selectel-na-fone-povyshennogo-sprosa-na-obligaczii-chetvertogo-vypuska-uvelichil-obem-razmeshheniya-do-4-mlrd-rublej/</x:v>
+      </x:c>
+      <x:c r="AB54" s="41" t="str">
+        <x:v>Selectel на фоне повышенного спроса на облигации четвертого выпуска увеличил объем размещения до 4 млрд рублей Компания Selectel сообщила об успешном закрытии книги заявок в рамках размещения четвертого выпуска облигаций. Объем выпуска составил 4 млрд рублей, ставка купона установлена на уровне 15% годовых с ежемесячной выплатой, срок обращения 2 года.</x:v>
+      </x:c>
+      <x:c r="AC54" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="41" t="str">
+        <x:v>DL-3b4a4419ab6b81bf</x:v>
+      </x:c>
+      <x:c r="B55" s="43" t="n">
+        <x:v>45357</x:v>
+      </x:c>
+      <x:c r="C55" s="41" t="str">
+        <x:v>DCM</x:v>
+      </x:c>
+      <x:c r="D55" s="41" t="str">
+        <x:v>Announced</x:v>
+      </x:c>
+      <x:c r="E55" s="41" t="str">
+        <x:v>SELECTEL</x:v>
+      </x:c>
+      <x:c r="F55" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="G55" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H55" s="41" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I55" s="44" t="n">
+        <x:v>3000000000</x:v>
+      </x:c>
+      <x:c r="J55" s="44"/>
+      <x:c r="K55" s="41" t="str">
+        <x:v>RUB</x:v>
+      </x:c>
+      <x:c r="L55" s="45"/>
+      <x:c r="M55" s="41" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="N55" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O55" s="44"/>
+      <x:c r="P55" s="44"/>
+      <x:c r="Q55" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R55" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S55" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J55&gt;0,$O55&gt;0,$K55=$R55),$J55/$O55,""),"")</x:f>
+      </x:c>
+      <x:c r="T55" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J55&gt;0,$P55&gt;0,$K55=$R55),$J55/$P55,""),"")</x:f>
+      </x:c>
+      <x:c r="U55" s="41" t="str">
+        <x:v>Bonds</x:v>
+      </x:c>
+      <x:c r="V55" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W55" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="X55" s="41" t="str">
+        <x:v>confirmed</x:v>
+      </x:c>
+      <x:c r="Y55" s="41" t="str"/>
+      <x:c r="Z55" s="41" t="str">
+        <x:v>Selectel Newsroom</x:v>
+      </x:c>
+      <x:c r="AA55" s="41" t="str">
+        <x:v>https://selectel.ru/about/newsroom/news/selectel-planiruet-razmeshhenie-obligaczij-obemom-3-milliarda-rublej/</x:v>
+      </x:c>
+      <x:c r="AB55" s="41" t="str">
+        <x:v>Selectel планирует размещение облигаций объемом 3 миллиарда рублей Selectel планирует разместить выпуск облигаций объемом 3 млрд рублей с фиксированной ставкой купона и сроком обращения 2 года. Ориентир доходности — премия не выше 275 базисных пунктов к значению кривой бескупонной доходности (КБД) Московской биржи на сроке 2 года. Купонные выплаты будут осуществляться ежемесячно. Сбор заявок планируется провести в первой декаде апреля.</x:v>
+      </x:c>
+      <x:c r="AC55" s="41" t="str">
+        <x:v>Screening record; verify against primary transaction documents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="41" t="str">
+        <x:v>DL-0242cf80b3f97c9c</x:v>
+      </x:c>
+      <x:c r="B56" s="43" t="n">
+        <x:v>45288</x:v>
+      </x:c>
+      <x:c r="C56" s="41" t="str">
+        <x:v>M&amp;A</x:v>
+      </x:c>
+      <x:c r="D56" s="41" t="str">
+        <x:v>Reported</x:v>
+      </x:c>
+      <x:c r="E56" s="41" t="str">
+        <x:v>25% провайдера IT-инфраструктуры Selectel Инвестиционный фонд Tier 5, основанный Геворком Вермишяном</x:v>
+      </x:c>
+      <x:c r="F56" s="41" t="str">
+        <x:v>Инвестиционный фонд Tier 5</x:v>
+      </x:c>
+      <x:c r="G56" s="41" t="str">
+        <x:v>Not classified</x:v>
+      </x:c>
+      <x:c r="H56" s="41" t="str">
+        <x:v>Russia</x:v>
+      </x:c>
+      <x:c r="I56" s="44"/>
+      <x:c r="J56" s="44"/>
+      <x:c r="K56" s="41" t="str">
+        <x:v>NOT DISCLOSED</x:v>
+      </x:c>
+      <x:c r="L56" s="45" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="M56" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="N56" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="O56" s="44"/>
+      <x:c r="P56" s="44"/>
+      <x:c r="Q56" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="R56" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="S56" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J56&gt;0,$O56&gt;0,$K56=$R56),$J56/$O56,""),"")</x:f>
+      </x:c>
+      <x:c r="T56" s="46" t="str">
+        <x:f>IFERROR(IF(AND($J56&gt;0,$P56&gt;0,$K56=$R56),$J56/$P56,""),"")</x:f>
+      </x:c>
+      <x:c r="U56" s="41" t="str">
+        <x:v>Acquisition / disposal</x:v>
+      </x:c>
+      <x:c r="V56" s="41" t="str">
+        <x:v>Not disclosed</x:v>
+      </x:c>
+      <x:c r="W56" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="X56" s="41" t="str">
+        <x:v>confirmed</x:v>
+      </x:c>
+      <x:c r="Y56" s="41" t="str"/>
+      <x:c r="Z56" s="41" t="str">
+        <x:v>Selectel Newsroom</x:v>
+      </x:c>
+      <x:c r="AA56" s="41" t="str">
+        <x:v>https://selectel.ru/about/newsroom/news/investicionnyj-fond-tier-5-priobrel-25-provajdera-it-infrastruktury-selectel/</x:v>
+      </x:c>
+      <x:c r="AB56" s="41" t="str">
+        <x:v>Инвестиционный фонд Tier 5 приобрел 25% провайдера IT-инфраструктуры Selectel Инвестиционный фонд Tier 5, основанный Геворком Вермишяном, ранее возглавлявшим «МегаФон», приобрел 25% провайдера IT-инфраструктуры Selectel, который входит в топ-3 российских IaaS-компаний по выручке. Детали сделки стороны не раскрывают.</x:v>
+      </x:c>
+      <x:c r="AC56" s="41" t="str">
         <x:v>Screening record; verify against primary transaction documents.</x:v>
       </x:c>
     </x:row>
@@ -4143,7 +5178,7 @@
     <x:mergeCell ref="A2:AC2"/>
     <x:mergeCell ref="A4:AC4"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="W7:W43">
+  <x:conditionalFormatting sqref="W7:W56">
     <x:cfRule type="colorScale" priority="1">
       <x:colorScale>
         <x:cfvo type="min"/>
@@ -4157,7 +5192,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R486e431c6e5f49cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f7c49853e947be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4196,7 +5231,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>DCM | Reported</x:v>
+        <x:v>DCM | Completed</x:v>
       </x:c>
       <x:c r="B4" s="9"/>
       <x:c r="C4" s="9"/>
@@ -4211,7 +5246,7 @@
         <x:v>Headline</x:v>
       </x:c>
       <x:c r="B6" s="55" t="str">
-        <x:v>О регистрации выпуска биржевых облигаций, о включении его в Список ценных бумаг, допущенных к торгам, и о присвоении указанным биржевым облигациям регистрационного номера</x:v>
+        <x:v>МТС успешно закрыла книгу биржевых облигаций 003Р-03 на 20 млрд руб.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4219,7 +5254,7 @@
         <x:v>Announced date</x:v>
       </x:c>
       <x:c r="B7" s="58" t="n">
-        <x:v>46199</x:v>
+        <x:v>46201</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4227,7 +5262,7 @@
         <x:v>Target / Issuer</x:v>
       </x:c>
       <x:c r="B8" s="56" t="str">
-        <x:v>Not disclosed</x:v>
+        <x:v>MTSS</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4242,7 +5277,9 @@
       <x:c r="A10" s="49" t="str">
         <x:v>Transaction value</x:v>
       </x:c>
-      <x:c r="B10" s="59"/>
+      <x:c r="B10" s="59" t="n">
+        <x:v>20000000000</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="49" t="str">
@@ -4255,7 +5292,7 @@
         <x:v>Currency</x:v>
       </x:c>
       <x:c r="B12" s="56" t="str">
-        <x:v>NOT DISCLOSED</x:v>
+        <x:v>RUB</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4329,7 +5366,7 @@
         <x:v>Evidence / score</x:v>
       </x:c>
       <x:c r="B22" s="56" t="str">
-        <x:v>confirmed / 7 out of 10</x:v>
+        <x:v>confirmed / 6 out of 10</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -4337,7 +5374,7 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B23" s="56" t="str">
-        <x:v>MOEX disclosure</x:v>
+        <x:v>MTS Investor Relations</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -4428,13 +5465,13 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="41" t="str">
-        <x:v>DL-moex-101492</x:v>
+        <x:v>DL-4d8f7bcb385b1c88</x:v>
       </x:c>
       <x:c r="B7" s="43" t="n">
-        <x:v>46199</x:v>
+        <x:v>46201</x:v>
       </x:c>
       <x:c r="C7" s="41" t="str">
-        <x:v>MOEX disclosure</x:v>
+        <x:v>MTS Investor Relations</x:v>
       </x:c>
       <x:c r="D7" s="41" t="str">
         <x:v>See Precedent Transactions → Source URL</x:v>
@@ -4443,12 +5480,12 @@
         <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F7" s="41" t="str">
-        <x:v>О регистрации выпуска биржевых облигаций, о включении его в Список ценных бумаг, допущенных к торгам, и о присвоении указанным биржевым облигациям регистрационного номера</x:v>
+        <x:v>МТС успешно закрыла книгу биржевых облигаций 003Р-03 на 20 млрд руб.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="41" t="str">
-        <x:v>DL-moex-101473</x:v>
+        <x:v>DL-moex-101492</x:v>
       </x:c>
       <x:c r="B8" s="43" t="n">
         <x:v>46199</x:v>
@@ -4463,12 +5500,12 @@
         <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F8" s="41" t="str">
-        <x:v>О регистрации проспекта биржевых облигаций</x:v>
+        <x:v>О регистрации выпуска биржевых облигаций, о включении его в Список ценных бумаг, допущенных к торгам, и о присвоении указанным биржевым облигациям регистрационного номера</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="41" t="str">
-        <x:v>DL-moex-101468</x:v>
+        <x:v>DL-moex-101473</x:v>
       </x:c>
       <x:c r="B9" s="43" t="n">
         <x:v>46199</x:v>
@@ -4483,12 +5520,12 @@
         <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F9" s="41" t="str">
-        <x:v>О регистрации изменений в эмиссионные документы</x:v>
+        <x:v>О регистрации проспекта биржевых облигаций</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="41" t="str">
-        <x:v>DL-moex-101457</x:v>
+        <x:v>DL-moex-101468</x:v>
       </x:c>
       <x:c r="B10" s="43" t="n">
         <x:v>46199</x:v>
@@ -4503,12 +5540,12 @@
         <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F10" s="41" t="str">
-        <x:v>О порядке сбора заявок и заключения сделок при размещении облигаций серии Б-1-403 Банк ВТБ (публичное акционерное общество) с 29 июня 2026 года</x:v>
+        <x:v>О регистрации изменений в эмиссионные документы</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="41" t="str">
-        <x:v>DL-moex-101454</x:v>
+        <x:v>DL-moex-101457</x:v>
       </x:c>
       <x:c r="B11" s="43" t="n">
         <x:v>46199</x:v>
@@ -4523,12 +5560,12 @@
         <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F11" s="41" t="str">
-        <x:v>О порядке приобретения облигаций серии 001P-04 ООО "АРЕНЗА-ПРО" с 29 июня 2026 год</x:v>
+        <x:v>О порядке сбора заявок и заключения сделок при размещении облигаций серии Б-1-403 Банк ВТБ (публичное акционерное общество) с 29 июня 2026 года</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="41" t="str">
-        <x:v>DL-moex-101451</x:v>
+        <x:v>DL-moex-101454</x:v>
       </x:c>
       <x:c r="B12" s="43" t="n">
         <x:v>46199</x:v>
@@ -4543,12 +5580,12 @@
         <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F12" s="41" t="str">
-        <x:v>О проведении выкупа облигаций с 29 июня по 03 июля 2026 года</x:v>
+        <x:v>О порядке приобретения облигаций серии 001P-04 ООО "АРЕНЗА-ПРО" с 29 июня 2026 год</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="41" t="str">
-        <x:v>DL-moex-101450</x:v>
+        <x:v>DL-moex-101451</x:v>
       </x:c>
       <x:c r="B13" s="43" t="n">
         <x:v>46199</x:v>
@@ -4563,67 +5600,67 @@
         <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F13" s="41" t="str">
-        <x:v>Дополнительные условия проведения торгов по выкупу облигаций серии 003Р-02 ООО "Концерн "РОССИУМ" 26 июня 2026 года</x:v>
+        <x:v>О проведении выкупа облигаций с 29 июня по 03 июля 2026 года</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="41" t="str">
-        <x:v>DL-bec65812ff9fcfae</x:v>
+        <x:v>DL-moex-101450</x:v>
       </x:c>
       <x:c r="B14" s="43" t="n">
-        <x:v>46197</x:v>
+        <x:v>46199</x:v>
       </x:c>
       <x:c r="C14" s="41" t="str">
-        <x:v>ComNews.ru</x:v>
+        <x:v>MOEX disclosure</x:v>
       </x:c>
       <x:c r="D14" s="41" t="str">
         <x:v>See Precedent Transactions → Source URL</x:v>
       </x:c>
       <x:c r="E14" s="41" t="str">
-        <x:v>unverified</x:v>
+        <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F14" s="41" t="str">
-        <x:v>Selectel разместит облигации на 5 млрд руб. для рефинансирования и инвестиций - ComNews.ru</x:v>
+        <x:v>Дополнительные условия проведения торгов по выкупу облигаций серии 003Р-02 ООО "Концерн "РОССИУМ" 26 июня 2026 года</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="41" t="str">
-        <x:v>DL-48bd4fc3fa031e6c</x:v>
+        <x:v>DL-bec65812ff9fcfae</x:v>
       </x:c>
       <x:c r="B15" s="43" t="n">
-        <x:v>46192</x:v>
+        <x:v>46197</x:v>
       </x:c>
       <x:c r="C15" s="41" t="str">
-        <x:v>Yandex Investor Relations</x:v>
+        <x:v>ComNews.ru</x:v>
       </x:c>
       <x:c r="D15" s="41" t="str">
         <x:v>See Precedent Transactions → Source URL</x:v>
       </x:c>
       <x:c r="E15" s="41" t="str">
-        <x:v>confirmed</x:v>
+        <x:v>unverified</x:v>
       </x:c>
       <x:c r="F15" s="41" t="str">
-        <x:v>Яндекс разместил два выпуска биржевых облигаций на общую сумму 60 млрд рублей</x:v>
+        <x:v>Selectel разместит облигации на 5 млрд руб. для рефинансирования и инвестиций - ComNews.ru</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="41" t="str">
-        <x:v>DL-9092ffd6a36a0a81</x:v>
+        <x:v>DL-7a721642a53e0f1d</x:v>
       </x:c>
       <x:c r="B16" s="43" t="n">
-        <x:v>46183</x:v>
+        <x:v>46192</x:v>
       </x:c>
       <x:c r="C16" s="41" t="str">
-        <x:v>Интерфакс</x:v>
+        <x:v>Yandex Investor Relations</x:v>
       </x:c>
       <x:c r="D16" s="41" t="str">
         <x:v>See Precedent Transactions → Source URL</x:v>
       </x:c>
       <x:c r="E16" s="41" t="str">
-        <x:v>unverified</x:v>
+        <x:v>confirmed</x:v>
       </x:c>
       <x:c r="F16" s="41" t="str">
-        <x:v>"Норникель" зафиксировал объем размещения облигаций на уровне 3 млрд юаней - Интерфакс</x:v>
+        <x:v>Яндекс разместил два выпуска биржевых облигаций на общую сумму 60 млрд рублей</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
@@ -4663,7 +5700,7 @@
         <x:v>Duplicate deal IDs</x:v>
       </x:c>
       <x:c r="B23" t="n">
-        <x:f>SUMPRODUCT(--(COUNTIF('Precedent Transactions'!$A$7:$A$43,'Precedent Transactions'!$A$7:$A$43)&gt;1))/2</x:f>
+        <x:f>SUMPRODUCT(--(COUNTIF('Precedent Transactions'!$A$7:$A$56,'Precedent Transactions'!$A$7:$A$56)&gt;1))/2</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C23" t="n">
@@ -4686,7 +5723,7 @@
         <x:v>Missing source URLs</x:v>
       </x:c>
       <x:c r="B24" t="n">
-        <x:f>COUNTBLANK('Precedent Transactions'!$AA$7:$AA$43)</x:f>
+        <x:f>COUNTBLANK('Precedent Transactions'!$AA$7:$AA$56)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C24" t="n">
@@ -4709,7 +5746,7 @@
         <x:v>Missing announced dates</x:v>
       </x:c>
       <x:c r="B25" t="n">
-        <x:f>COUNTBLANK('Precedent Transactions'!$B$7:$B$43)</x:f>
+        <x:f>COUNTBLANK('Precedent Transactions'!$B$7:$B$56)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C25" t="n">
@@ -4732,7 +5769,7 @@
         <x:v>Unsafe / non-HTTP URLs</x:v>
       </x:c>
       <x:c r="B26" t="n">
-        <x:f>SUMPRODUCT(--(LEFT('Precedent Transactions'!$AA$7:$AA$43,4)&lt;&gt;"http"),--('Precedent Transactions'!$A$7:$A$43&lt;&gt;""))</x:f>
+        <x:f>SUMPRODUCT(--(LEFT('Precedent Transactions'!$AA$7:$AA$56,4)&lt;&gt;"http"),--('Precedent Transactions'!$A$7:$A$56&lt;&gt;""))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C26" t="n">
@@ -4755,15 +5792,15 @@
         <x:v>Missing target / issuer</x:v>
       </x:c>
       <x:c r="B27" t="n">
-        <x:f>COUNTIF('Precedent Transactions'!$E$7:$E$43,"Not disclosed")</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTIF('Precedent Transactions'!$E$7:$E$56,"Not disclosed")</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C27" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D27" t="n">
         <x:f>B27-C27</x:f>
-        <x:v>20</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E27" t="n">
         <x:v>0</x:v>
@@ -4778,7 +5815,7 @@
         <x:v>EV without revenue/EBITDA</x:v>
       </x:c>
       <x:c r="B28" t="n">
-        <x:f>SUMPRODUCT(--('Precedent Transactions'!$J$7:$J$43&gt;0),--('Precedent Transactions'!$O$7:$O$43=""),--('Precedent Transactions'!$P$7:$P$43=""))</x:f>
+        <x:f>SUMPRODUCT(--('Precedent Transactions'!$J$7:$J$56&gt;0),--('Precedent Transactions'!$O$7:$O$56=""),--('Precedent Transactions'!$P$7:$P$56=""))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C28" t="n">
@@ -4801,7 +5838,7 @@
         <x:v>Multiple without enterprise value</x:v>
       </x:c>
       <x:c r="B29" t="n">
-        <x:f>SUMPRODUCT(--('Precedent Transactions'!$J$7:$J$43=""),--((('Precedent Transactions'!$S$7:$S$43&gt;0)+('Precedent Transactions'!$T$7:$T$43&gt;0))&gt;0))</x:f>
+        <x:f>SUMPRODUCT(--('Precedent Transactions'!$J$7:$J$56=""),--((('Precedent Transactions'!$S$7:$S$56&gt;0)+('Precedent Transactions'!$T$7:$T$56&gt;0))&gt;0))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C29" t="n">

</xml_diff>

<commit_message>
chore: refresh deal desk
</commit_message>
<xml_diff>
--- a/output/precedent_transactions.xlsx
+++ b/output/precedent_transactions.xlsx
@@ -23,7 +23,7 @@
     <t>DEAL MARKETS COPILOT — SUMMARY</t>
   </si>
   <si>
-    <t>As of 2026-07-02 | Build a4432f860b74 | Quality-controlled transaction monitor</t>
+    <t>As of 2026-07-03 | Build a4432f860b74 | Quality-controlled transaction monitor</t>
   </si>
   <si>
     <t>DATABASE SNAPSHOT</t>
@@ -6742,13 +6742,10 @@
         <v>237</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="K49" s="8">
-        <v>35000000000</v>
+        <v>70</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>70</v>
@@ -11567,7 +11564,7 @@
         <v>258</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>70</v>

</xml_diff>